<commit_message>
9th Commit : Appium Server Connection Established
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD5F093-C7FB-4077-9FBF-20D6CCCC7834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DC816F-5F18-4F9B-889E-B836CCE9D622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="AddCustomer" sheetId="13" r:id="rId2"/>
-    <sheet name="AddCityArea" sheetId="1" r:id="rId3"/>
-    <sheet name="AddCityAdmin" sheetId="2" r:id="rId4"/>
-    <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
-    <sheet name="AddBikeDriver" sheetId="4" r:id="rId6"/>
-    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId7"/>
-    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId8"/>
-    <sheet name="AddStore" sheetId="7" r:id="rId9"/>
-    <sheet name="StoreOperations" sheetId="8" r:id="rId10"/>
-    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId11"/>
-    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId12"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
-    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
-    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId15"/>
-    <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId16"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId17"/>
+    <sheet name="UniversalFlow" sheetId="31" r:id="rId2"/>
+    <sheet name="AddCustomer" sheetId="13" r:id="rId3"/>
+    <sheet name="AddCityArea" sheetId="1" r:id="rId4"/>
+    <sheet name="AddCityAdmin" sheetId="2" r:id="rId5"/>
+    <sheet name="AddAutoDriver" sheetId="3" r:id="rId6"/>
+    <sheet name="AddBikeDriver" sheetId="4" r:id="rId7"/>
+    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId8"/>
+    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId9"/>
+    <sheet name="AddStore" sheetId="7" r:id="rId10"/>
+    <sheet name="StoreOperations" sheetId="8" r:id="rId11"/>
+    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId12"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId13"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId14"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId15"/>
+    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId16"/>
+    <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId17"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId18"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="113">
   <si>
     <t>City Area</t>
   </si>
@@ -3095,6 +3096,28 @@
 176.Click  Submit,click,,"//button[normalize-space()='Submit']"
 177.Verify Sucess, verify, , "//div[@aria-label='Info']"
 178.wait,2000,,</t>
+  </si>
+  <si>
+    <t>SA_TS_33</t>
+  </si>
+  <si>
+    <t>UniversalFlow</t>
+  </si>
+  <si>
+    <t>TC_CA_00_Universal_Flow</t>
+  </si>
+  <si>
+    <t>UniversalFlow is verified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Load Site,navigate,https://dev.we1.co/#/login,
+2.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
+3.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
+4.Click Login,click,,"//button[@type='submit']"
+5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
+6.Load User App,switch_to,user,
+7.wait,5000,,
+</t>
   </si>
 </sst>
 </file>
@@ -3542,6 +3565,78 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3613,7 +3708,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3685,7 +3780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73960651-1493-478A-BEDA-A31CF297E315}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3757,7 +3852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3829,7 +3924,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3901,7 +3996,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6277B-DBCF-4BFF-819C-1E90748D3258}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3973,7 +4068,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6B7FC7-76CD-491F-AC51-1837B3B068AC}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4038,7 +4133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4113,6 +4208,82 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1717BC20-9348-4B52-9588-34F52BC8B75D}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="36.88671875" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4188,7 +4359,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4264,7 +4435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4329,7 +4500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4401,7 +4572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4197A722-266E-4219-9B46-8F4D56D7D7A1}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4473,7 +4644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790BFFF3-3BE5-4068-A6FF-6214BEDD72BA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4545,7 +4716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DB4E5D-EBF5-4B6A-BF83-7934D70C5535}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4616,76 +4787,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
10th Commit : Mobile Integration Done In ABCD Framework
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DC816F-5F18-4F9B-889E-B836CCE9D622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD6CB3B-5825-4CF5-A965-E0EFF5DB6800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3110,14 +3110,15 @@
     <t>UniversalFlow is verified</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Load Site,navigate,https://dev.we1.co/#/login,
+    <t>1.Load Site,navigate,https://dev.we1.co/#/login,
 2.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
 3.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
 4.Click Login,click,,"//button[@type='submit']"
 5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
 6.Load User App,switch_to,user,
 7.wait,5000,,
-</t>
+8.Load Driver App,switch_to,driver,
+9.wait,5000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
11th Commit : Mobile Integration Succsessfull In ABCD Framework
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD6CB3B-5825-4CF5-A965-E0EFF5DB6800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EC1EA8-2C6E-4EC3-94A5-E0208F982DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3110,15 +3110,19 @@
     <t>UniversalFlow is verified</t>
   </si>
   <si>
-    <t>1.Load Site,navigate,https://dev.we1.co/#/login,
+    <t xml:space="preserve">1.Load Site,navigate,https://dev.we1.co/#/login,
 2.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
 3.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
 4.Click Login,click,,"//button[@type='submit']"
 5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
 6.Load User App,switch_to,user,
 7.wait,5000,,
-8.Load Driver App,switch_to,driver,
-9.wait,5000,,</t>
+8.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+9.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.wait,3000,,
+10.Load Driver App,switch_to,driver,
+11.wait,5000,,
+</t>
   </si>
 </sst>
 </file>
@@ -4249,7 +4253,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>108</v>
       </c>

</xml_diff>

<commit_message>
61th Commit : Customer Locator Added
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E21B82-E5FC-4236-BA48-8107482CD04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3ACB132-3CED-47AB-9032-CAFCB3B4D90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="AddCustomer" sheetId="13" r:id="rId2"/>
+    <sheet name="AddCustomer" sheetId="31" r:id="rId2"/>
     <sheet name="AddCityArea" sheetId="1" r:id="rId3"/>
     <sheet name="AddCityAdmin" sheetId="2" r:id="rId4"/>
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
@@ -110,12 +110,6 @@
   </si>
   <si>
     <t>TC_CA_00_super_admin_login</t>
-  </si>
-  <si>
-    <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-2. Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-3. Click Login,click,,"//button[@type='submit']"
-4. Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"</t>
   </si>
   <si>
     <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
@@ -1746,88 +1740,6 @@
   </si>
   <si>
     <t>This test case validates the end-to-end management of subscription plan architectures across four distinct user entities: Store, Driver, Provider, and Customer. The workflow systematically executes the creation of localized "Premium" plans for various service categories—such as Food Delivery and Pest Control—featuring integrated multi-language support in Arabic, Tamil, and Hindi. The validation cycle spans from defining plan durations, pricing, and free-ride quotas to conducting administrative audits including localized description verification, active/inactive state toggling, and data filtering. The process concludes by confirming the operational lifecycle through record modification and final deletion, ensuring the functional stability and localized integrity of the platform’s commercial monetization modules.</t>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-20.Click Close, click, , "//button[normalize-space()='Close']"
-21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
-22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-26.Click Submit, click, , "//button[normalize-space()='Submit']"
-27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-32.Click Submit, click, , "//button[normalize-space()='Submit']"
-33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-36.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
-41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
-46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
-47.Click Submit, click, , "//button[normalize-space()='Submit']"
-48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
-54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
-55.Click Submit, click, , "//button[normalize-space()='Submit']"
-56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-59.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-63.Click Disable  Icon,click,,"//i[@title='Block']"
-64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
-65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
-66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked Customers']"
-71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
-73.Click Enable  Icon,click,,"//i[@title='Status']"
-74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
-75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-77.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-80.wait,1000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
@@ -3095,6 +3007,93 @@
 42. Verify Success Message,verify,,"//div[@aria-label='Info']"
 43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
 </t>
+  </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "admin.login.email"
+2. Enter Password,type,R1mep@321, "admin.login.password"
+3. Click Login,click,,"admin.login.submit_btn"
+4. Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
+  </si>
+  <si>
+    <t>1. Click Customer Icon,click,,"admin.menu.customer_icon"
+2.Click Add Customers,click,,"admin.menu.add_customers"
+3. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
+4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "admin.customer.input_name"
+5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "admin.customer.input_email"
+6.Enter Contact Number, type, {randomPhone}, "admin.customer.input_phone"
+7.Enter Video Call Limit, type, 60, "admin.customer.input_video_limit"
+8.Open Gender,click,,"admin.customer.dropdown_gender"
+9.Select Male,click,,"admin.customer.select_gender_male"
+10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "admin.customer.upload_profile_img"
+11.Click Submit, click, , "admin.customer.submit_btn"
+12.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+13. Click Customer Icon,click,,"admin.menu.customer_icon"
+14. Click Customer Icon,click,,"admin.menu.customer_icon"
+15.Click Verified Customers,click,,"admin.menu.verified_customers"
+16. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+17.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+18.Scroll Grid, tab, 7, "admin.customer.filter_name"
+19.Click Edit Icon ,click,,"admin.customer.grid.btn_edit"
+20.Click Close, click, , "admin.customer.grid.btn_close"
+21.Click Wallet Icon ,click,,"admin.customer.grid.btn_wallet"
+22.Click Add Money ,click,,"admin.customer.wallet.btn_add_money"
+23.Enter Wallet Amount, type, 1000, "admin.customer.wallet.input_amount"
+24.Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
+25.Select Add Money,click,,"admin.customer.wallet.select_add_money"
+26.Click Submit, click, , "admin.customer.submit_btn"
+27.Verify Saved Succesfully, verify, , "admin.customer.toast_added_success"
+28.Click Add Money ,click,,"admin.customer.wallet.btn_add_money"
+29.Enter Wallet Amount, type, 200, "admin.customer.wallet.input_amount"
+30.Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
+31.Select Deduct Money,click,,"admin.customer.wallet.select_deduct_money"
+32.Click Submit, click, , "admin.customer.submit_btn"
+33.Verify Saved Succesfully, verify, , "admin.customer.toast_added_success"
+34. Click Customer Icon,click,,"admin.menu.customer_icon"
+35. Click Customer Icon,click,,"admin.menu.customer_icon"
+36.Click Verified Customers,click,,"admin.menu.verified_customers"
+37. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+38.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+39.Scroll Grid, tab, 7, "admin.customer.filter_name"
+40.Click Loyalty Points Icon,click,,"admin.customer.grid.btn_loyalty_points"
+41.Click Manage Loyality Points, click, , "admin.customer.loyalty.btn_manage"
+42.Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
+43.Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
+44.Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
+45.Select Add Points,click,,"admin.customer.loyalty.select_add_points"
+46.Enter Points, type, 30, "admin.customer.loyalty.input_points"
+47.Click Submit, click, , "admin.customer.submit_btn"
+48.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+49.Click Manage Loyality Points, click, , "admin.customer.loyalty.btn_manage"
+50.Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
+51.Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
+52.Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
+53.Select Deduct Points,click,,"admin.customer.loyalty.select_deduct_points"
+54.Enter Points, type, 10, "admin.customer.loyalty.input_points"
+55.Click Submit, click, , "admin.customer.submit_btn"
+56.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+57. Click Customer Icon,click,,"admin.menu.customer_icon"
+58. Click Customer Icon,click,,"admin.menu.customer_icon"
+59.Click Verified Customers,click,,"admin.menu.verified_customers"
+60. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+61.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+62.Scroll Grid, tab, 7, "admin.customer.filter_name"
+63.Click Disable Icon,click,,"admin.customer.grid.btn_block"
+64.Click Disable User Yes,click,,"admin.customer.dialog.btn_confirm_yes"
+65.Disable Reason,type,Client Complaints,"admin.customer.dialog.textarea_reason"
+66.Click Reject Yes,click,,"admin.customer.dialog.btn_confirm_yes"
+67.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+68. Click Customer Icon,click,,"admin.menu.customer_icon"
+69. Click Customer Icon,click,,"admin.menu.customer_icon"
+70.Click Blocked Customers,click,,"admin.menu.blocked_customers"
+71.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+72.Scroll Grid, tab, 10, "admin.customer.filter_name"
+73.Click Enable Icon,click,,"admin.customer.grid.btn_status_enable"
+74.Click Enable Yes,click,,"admin.customer.dialog.btn_confirm_yes"
+75. Click Customer Icon,click,,"admin.menu.customer_icon"
+76. Click Customer Icon,click,,"admin.menu.customer_icon"
+77.Click Verified Customers,click,,"admin.menu.verified_customers"
+78. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+79.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
   </si>
 </sst>
 </file>
@@ -3511,19 +3510,19 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3583,22 +3582,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3655,22 +3654,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3727,22 +3726,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3799,22 +3798,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3871,22 +3870,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3943,22 +3942,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4015,22 +4014,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4080,22 +4079,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4113,7 +4112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4396F6CA-D57B-49F5-A8ED-CEBB93A6ED43}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4158,19 +4157,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4237,16 +4236,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4312,16 +4311,16 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -4377,16 +4376,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4449,16 +4448,16 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4515,22 +4514,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4587,22 +4586,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4660,22 +4659,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
69th Commit: Tranport Sevice Locator File Created
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34816D78-B912-4358-B4A5-4C37AB9A8B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106C96A7-C8B0-4924-B6A1-AEF71A3DCFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="AddAutoDriver" sheetId="33" r:id="rId5"/>
     <sheet name="AddBikeDriver" sheetId="34" r:id="rId6"/>
     <sheet name="AddTaxiDriver" sheetId="35" r:id="rId7"/>
-    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId8"/>
+    <sheet name="TransportServiceCompleteTest" sheetId="37" r:id="rId8"/>
     <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId9"/>
     <sheet name="AddStore" sheetId="7" r:id="rId10"/>
     <sheet name="StoreOperations" sheetId="8" r:id="rId11"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="114">
   <si>
     <t>City Area</t>
   </si>
@@ -1740,186 +1740,6 @@
   </si>
   <si>
     <t>Super Admin Login</t>
-  </si>
-  <si>
-    <t>1.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-2. Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-3.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-4.Click  Add Category,click,,"//button[normalize-space()='Add Category']"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "//input[@placeholder='Service Name (in Arabic)']"
-7.Enter Slug, type, Bus Ride, "//input[@placeholder='Slug']"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "//input[@type='file' and @accept='image/*']"
-9.wait,2000,,
-10.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-11.Select Activate,click,,"//li[@aria-label='Activate']"
-12.Open Select City Dropdown,click,,"//span[text()='Select City']/ancestor::app-drop-down//div[contains(@class, 'p-multiselect-label-container')]"
-13.Select {areaName},click,,"//li[@aria-label='{areaName}']"
-14.Click  Submit,click,,"//button[normalize-space()='Submit']"
-15.Verify Sucess, verify, , "//div[@aria-label='Info']"
-16.wait,2000,,
-17.Click  back,click,,"//button[normalize-space()='Back']"
-18.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-19.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-20.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-21.Click Home Icon ,click,,"//i[@title='Home']"
-22.Click Settings ,click,,"//button[contains(., 'Settings')]"
-23.Click Vehicle Type,click,,"//div[normalize-space()='Vehicle Type']"
-24.Click Add Vehicle Type,click,,"//button[normalize-space()='Add Vehicle Type']"
-25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "//input[@placeholder='Enter Vehicle Type']"
-26.Enter Base Fare, type, 150, "//input[@placeholder='Enter base fare']"
-27.Enter Base Fare Max Kilometer, type, 10, "//input[@placeholder='Enter Base Fare KM Limit']"
-28.Open Extra Distance Fare Dropdown,click,"//label[contains(., 'Extra Distance Fare Type')]/following-sibling::p-dropdown"
-29.Select Amount,click,,"//li[@aria-label='Amount']"
-30.Enter Extra Distance Fare , type, 10, "//input[@placeholder='Extra Distance Fare (Per Km)']"
-31.Enter Free Waiting Time , type, 10, "//label[contains(., 'Free Waiting Time')]/following::input[1]"
-32.Open Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[1])"
-33.Select Amount,click,,"//li[@aria-label='Amount']"
-34.Enter Waiting Rate , type, 10, "//input[@placeholder='Waiting Rate (per min)']"
-35.Enter Included Trip Waiting , type, 10, "//input[@placeholder='Included Trip Waiting']"
-36.Open Trip Waiting Charge Dropdown,click,"((//label[contains(., 'Waiting Charge Type')]/following::p-dropdown)[2])"
-37.Select Amount,click,,"//li[@aria-label='Amount']"
-38.Enter Trip Waiting Rate , type,50, "//input[@placeholder='Trip Waiting Rate (per min)']"
-39.Enter Free Pickup Distance , type,5, "//input[@placeholder='Free Pickup Distance (In kms)']"
-40.Open Pickup Charge Dropdown,click,"//label[contains(., 'Pickup Charge Type')]/following-sibling::p-dropdown"
-41.Select Amount,click,,"//li[@aria-label='Amount']"
-42.Enter Pickup Fee, type,50, "//input[@placeholder='Pickup Fee (Per Km)']"
-43.Open Customer Fee  Dropdown,click,"//span[@aria-label='Customer Fee Type']"
-44.Select Amount,click,,"//li[@aria-label='Amount']"
-45.Enter Customer Fee, type,50, "//input[@placeholder='Customer Fee']"
-46.Open Customer GST  Dropdown,click,"//label[contains(., 'Customer GST type')]/following-sibling::p-dropdown"
-47.Select Amount,click,,"//li[@aria-label='Amount']"
-48.Enter  GST amount, type,50, "//input[contains(@placeholder,'Enter GST amount or percentage')]"
-49.Open Driver Fee  Dropdown,click,"//span[@aria-label='Driver Fee Type']"
-50.Select Amount,click,,"//li[@aria-label='Amount']"
-51.Enter  Driver Fee, type,50, "//input[@placeholder='Driver Fee']"
-52.Open Driver GST  Dropdown,click,"//label[contains(., 'Driver GST type')]/following-sibling::p-dropdown"
-53.Select Amount,click,,"//li[@aria-label='Amount']"
-54.Enter Driver Gst,type,50," //input[@placeholder='Driver GST in amount or percentage']"
-55.Open Status Dropdown,click,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-56.Select Active,click,,"//li[@aria-label='Active']"
-57.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "//app-image-upload//input[@type='file' and @accept='image/*']"
-58.Enter Notifiacation,type,50,"//input[@placeholder='User will be notified when pickup km exceeds this']"
-59.Enter Driver Request ETA,type,50,"//input[@placeholder='Enter Driver ETA Limit']"
-60.Enter Driver Request KM,type,50,"//input[@placeholder='Driver Request KM Limit']"
-61.Click Surcharge Time Checkbox, click, , "//div[text()='EveryDay']/preceding-sibling::mat-checkbox"
-62.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
-63.Enter To Time, type, 220000PM, "((//input[@placeholder='--:--:-- --'])[2])"
-64.Open  Dropdown,click,"((//span[@aria-label='select type'])[1])"
-65.Select Amount,click,,"//li[@aria-label='Amount']"
-66.Enter  Price, type,50, "//input[@placeholder='Enter Price']"
-67.Click  Submit,click,,"//button[normalize-space()='Submit']"
-68.Verify Sucess, verify, , "//div[@aria-label='Info']"
-69.Click Settings ,click,,"//button[contains(., 'Settings')]"
-70.Click Promocode,click,,"//div[normalize-space()='Promocode']"
-71.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-72.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-73.Select User,click,,"//li[@aria-label='{customerName}']"
-74.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-75.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "//input[@placeholder='Code Name']"
-76.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-77.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-78.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-79.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-80.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-81.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-82.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-83.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-84.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-85.Click Submit ,click,,"//button[normalize-space()='Submit']"
-86.Verify Sucess, verify, , "//div[@aria-label='Info']"
-87.wait,2000,,
-88.Click Settings ,click,,"//button[contains(., 'Settings')]"
-89.Click Service Settings ,click,,"//div[normalize-space()='Service Setting']"
-90.Enter Driver Accept Timeout, type, 60, "//label[contains(., "Driver Accept Timeout")]/following::input[1]"
-91.Enter Driver Serach Radius, type, 50, "//label[contains(., "Driver Search Radius")]/following::input[1]"
-92.Click Submit ,click,,"//button[normalize-space()='Submit']"
-93.Verify Sucess, verify, , "//div[@aria-label='Info']"
-94.wait,1000,,
-95.Click Settings ,click,,"//button[contains(., 'Settings')]"
-96.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-97.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-98.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "//label[contains(., 'Name')]/following::input[1]"
-99.Open status Dropdown,click,,"//label[contains(., 'Status')]/following::div[contains(@class, 'p-dropdown')]"
-100.Select Active,click,,"//li[@aria-label='Active']"
-101.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-102.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-103.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-104.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-105.Click Submit ,click,,"//button[normalize-space()='Submit']"
-106.Verify Sucess, verify, , "//div[@aria-label='Info']"
-107.Filter Document List,type,{documentName},"//input[@aria-label='Name Filter Input']"
-108.wait,1000,,
-109.Click Settings ,click,,"//button[contains(., 'Settings')]"
-110.Click Customer Loyalty Settings,click,,"//div[text()=' Customer Loyalty Settings ']"
-111.Open status Allow Customer loyalty points,click,,"//label[contains(., 'Allow Customer loyalty points')]/following::div[contains(@class, 'p-dropdown')]"
-112.Select ON,click,,"//li[@role='option']//span[text()='ON']"
-113.Enter Minimum order amount for eligibility to redeem loyalty points, type, 100,"//label[contains(., 'Minimum order amount for eligibility to redeem loyalty points')]/following::input[1]"
-114.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10,"//label[contains(., 'Loyalty points redeem per order (in %) (% of order amount)')]/following::input[1]"
-115.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5,"//label[contains(., 'Loyalty points per default currency (for ex. $1 = 10 points)')]/following::input[1]"
-116.Click Submit ,click,,"//button[normalize-space()='Submit']"
-117.Verify Sucess, verify, , "//div[@aria-label='Info']"
-118.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-119.Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-120.Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-121.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-122.Select Bus Ride Option,click,,"//span[normalize-space()='{transportName}']"
-123.Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-124.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "//label[contains(.,'Full Name')]/following::input[1]"
-125.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "//label[contains(.,'Email')]/following::input[1]"
-126.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-127.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "//input[@type='file']"
-128.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-129.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-130.Select  volvo Option,click,,"//li[@role='option']//span[text()='{busTypeName}']"
-131.Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-132.Enter Vehicle Company, type, busCompany{randomAlpha}&gt;&gt; busCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-133.Enter Plate No, type, KL-01-AB-1634, "//label[contains(.,'Plate No')]/following::input[1]"
-134. Enter Model Name, type, deisel, "//label[contains(.,'Model Name')]/following::input[1]"
-135.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "(//input[@type='file'])[2]"
-136. Enter Vehicle Color, type, white, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-137.Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-138.Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-139.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-140.Enter Account Holder Name, type, {busDriverName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-141.Enter Payment Email Address, type, {busEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-142.Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-143.Click Submit, click, , "//button[contains(.,'Submit')]"
-144.Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-145.Wait for Toast to hide, wait, 1000,
-146.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-147.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-148.Click Pending Documents,click,," //span[normalize-space()='Pending Documents']"
-149.Filter by Name,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-150.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-151.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-152.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-153.FilterDocumet List,type,{documentName},"//input[@aria-label='Document Name Filter Input']"
-154.Add Driving License,click,,"//i[@title='Edit']"
-155.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-156.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-157.Click Submit, click, , "//button[normalize-space()='Submit']"
-158.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-159.Click Approve Driver,click,,"//i[@title='Approve']"
-160.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-161.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-162.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-163.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-164.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-165.Filter Approved Driver,type,{busDriverName},"//input[@aria-label='Driver Name Filter Input']"
-166.Click Transports Services Icon,click,,"//i[@class='fa-motorcycle fa-solid iconstyle']"
-167.Click Transports Services Menu,click,,"//h2[normalize-space()='Transport Services']"
-168.Verify Transport Services,verify,,"//div[normalize-space()='TRANSPORT SERVICES']"
-169.Filter Services List,type,{transportName},"//input[@aria-label='Services Filter Input']"
-170.Click Edit Icon ,click,,"//i[@title='Edit']"
-171.wait,2000,,
-172.Scroll Grid, tab, 5, "//input[@placeholder='Service Name']"
-173.wait,2000,,
-174.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-175.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-176.Click  Submit,click,,"//button[normalize-space()='Submit']"
-177.Verify Sucess, verify, , "//div[@aria-label='Info']"
-178.wait,2000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
@@ -2745,86 +2565,6 @@
 4.Load Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click Setting menu,click,,"web.global.menu.settings"
-3. Click City area menu,click,,"admin.menu.city_area"
-4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
-5. Click Add City Area button,click,,"admin.city_area.btn_add"
-6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
-7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
-8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
-9. Select Active,click,,"admin.city_area.select_status_active"
-10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
-11. wait,1000,,
-12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
-13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
-14. wait,1000,,
-15. Map Polygon,draw polygon,"-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120","//div[@class='ol-layer']//canvas"
-16. Click Submit,click,,"web.global.action.submit"
-17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
-18. Click Transport Services,click,,"admin.transport.card_link"
-19. Wait For Transport Page,wait_until_visible,,"admin.transport.page_heading"
-20. Click Add Category,click,,"admin.transport.btn_add_category"
-21. Open Select City Dropdown,click,,"admin.transport.dropdown_city_multiselect"
-22. Search City Area,type,{areaName},"admin.transport.input_filter_city"
-23. Verify Area in Dropdown,verify,,"admin.transport.select_filtered_option"
-24. Click close,click,,"web.global.action.close"
-25.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-26. Click Setting menu,click,,"web.global.menu.settings"
-27. Click City admin menu,click,,"admin.menu.city_admin"
-28. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
-29. Click Add City Admin button,click,,"admin.city_admin.btn_add"
-30. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
-31. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
-32. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
-</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click Setting menu,click,,web.global.menu.settings
-3. Click City admin menu,click,,admin.menu.city_admin
-4. Wait For City Admin List,wait_until_visible,,admin.city_admin.list_heading
-5. Click Add City Admin button,click,,admin.city_admin.btn_add
-6. Wait For Admin heading,wait_until_visible,,admin.city_admin.add_heading
-7.Select Name field,click,,admin.city_admin.input_name
-8. Enter Admin Name,type,faizal{randomAlpha} &gt;&gt; adminName,admin.city_admin.input_name
-9.Select Email field,click,,admin.city_admin.input_email
-10. Enter Email,type,faizal_{timestamp}@gmail.com,admin.city_admin.input_email
-11.select the password field,click,,admin.city_admin.input_password
-12.Enter the Password as "faizal@123",type,faizal@123,admin.city_admin.input_password
-13.Open Select City Dropdown,click,,admin.city_admin.select_city_dropdown
-14.Select {areaName},click,,admin.city_admin.select_dynamic_option
-15. Click on the "Transport Service" → "Auto Ride" checkbox,click,,admin.city_admin.chk_transport_autoride
-16.Click on the "Customers" → "Add Customers" checkbox,click,,admin.city_admin.chk_customer_add
-17.Click on the "Customers" → "Verified Customers"checkbox,click,,admin.city_admin.chk_customer_verified
-18.Click on the "Customers" → "Non Verified Customers" checkbox,click,,admin.city_admin.chk_customer_unverified
-19.Click on the "Customers" → "Blocked Customers" checkbox,click,,admin.city_admin.chk_customer_blocked
-20.Click on the "Customers" → "Deleted Customers" checkbox,click,,admin.city_admin.chk_customer_deleted
-21.Click on the "Customers" → "Pending Customers" checkbox,click,,admin.city_admin.chk_customer_pending
-22.Click on the "Providers" → "Transport Providers List" checkbox,click,,admin.city_admin.chk_provider_list
-23.Click on the "Drivers" → "Add Driver" checkbox,click,,admin.city_admin.chk_driver_add
-24.Click on the "Drivers" → "Approved Drivers" checkbox,click,,admin.city_admin.chk_driver_approved
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox,click,,admin.city_admin.chk_driver_unapproved
-26.Click on the "Drivers" → "Blocked Drivers" checkbox,click,,admin.city_admin.chk_driver_blocked
-27.Click on the "Drivers" → "Reject Drivers" checkbox,click,,admin.city_admin.chk_driver_rejected
-28.Click on the "Drivers" → "Deleted Drivers" checkbox,click,,admin.city_admin.chk_driver_deleted
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox,click,,admin.city_admin.chk_subscription_plan
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox,click,,admin.city_admin.chk_cashout
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox,click,,admin.city_admin.chk_report_customer
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox,click,,admin.city_admin.chk_report_driver
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,admin.city_admin.chk_report_provider
-34.Click on the "Report Issue" → "Report issue settings" checkbox,click,,admin.city_admin.chk_report_settings
-35.Click on the "Report Issue" → "FAQs" checkbox,click,,admin.city_admin.chk_report_faqs
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox,click,,admin.city_admin.chk_web_header_footer
-37.Click on the "Website Settings" → "Home Page Settings" checkbox,click,,admin.city_admin.chk_web_homepage
-38.Click on the "Website Settings" → "Delivery Settings" checkbox,click,,admin.city_admin.chk_web_delivery
-39.Click on the "Website Settings" → "Transport Settings" checkbox,click,,admin.city_admin.chk_web_transport
-40.Click on the "Website Settings" → "FAQs" checkbox,click,,admin.city_admin.chk_web_faqs
-41.Click Submit,click,,web.global.login.submit_btn
-42. Wait For Success Message,wait_until_visible,,web.global.toast.info
-43.Filter admin name,type,{adminName},admin.city_admin.input_name_filter</t>
-  </si>
-  <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click Customer Icon,click,,"admin.menu.customer_icon"
 3. Click Add Customers,click,,"admin.menu.add_customers"
@@ -3109,6 +2849,282 @@
     <t>7.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 8.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
 9.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,"web.global.menu.settings"
+3. Click City area menu,click,,"admin.menu.city_area"
+4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
+5. Click Add City Area button,click,,"admin.city_area.btn_add"
+6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
+7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
+8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
+9. Select Active,click,,"admin.city_area.select_status_active"
+10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
+11. wait,1000,,
+12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
+13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
+14. wait,1000,,
+15. Map Polygon,draw polygon,"-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120","//div[@class='ol-layer']//canvas"
+16. Click Submit,click,,"web.global.action.submit"
+17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
+18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+19. Click Transport Services,click,,"admin.transport.menu.card"
+20. Wait For Transport Page,wait_until_visible,,"admin.transport.page.header"
+21. Click Add Category,click,,"admin.transport.add_category.btn"
+22. Open Select City Dropdown,click,,"admin.transport.city.dropdown"
+23. Search City Area,type,{areaName},"admin.transport.input_filter_city"
+24. Verify Area in Dropdown,verify,,"admin.transport.city.dynamic_option"
+25. Click close,click,,"web.global.action.close"
+26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+27. Click Setting menu,click,,"web.global.menu.settings"
+28. Click City admin menu,click,,"admin.menu.city_admin"
+29. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+30. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+31. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+32. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+33. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
+</t>
+  </si>
+  <si>
+    <t>Removed Test Cases</t>
+  </si>
+  <si>
+    <t>21.Click on the "Customers" → "Pending Customers" checkbox,click,,admin.city_admin.chk_customer_pending
+35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox,click,,admin.city_admin.chk_web_header_footer
+36.Click on the "Website Settings" → "Home Page Settings" checkbox,click,,admin.city_admin.chk_web_homepage
+37.Click on the "Website Settings" → "Delivery Settings" checkbox,click,,admin.city_admin.chk_web_delivery
+38.Click on the "Website Settings" → "Transport Settings" checkbox,click,,admin.city_admin.chk_web_transport
+39.Click on the "Website Settings" → "FAQs" checkbox,click,,admin.city_admin.chk_web_faqs</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,"web.global.menu.settings"
+3. Click City admin menu,click,,"admin.menu.city_admin"
+4. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+5. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+6. Wait For Admin heading,wait_until_visible,,"admin.city_admin.add_heading"
+7.Select Name field,click,,"admin.city_admin.input_name"
+8. Enter Admin Name,type,faizal{randomAlpha} &gt;&gt; adminName,"admin.city_admin.input_name"
+9.Select Email field,click,,"admin.city_admin.input_email"
+10. Enter Email,type,faizal_{timestamp}@gmail.com,"admin.city_admin.input_email"
+11.select the password field,click,,"admin.city_admin.input_password"
+12.Enter the Password as "faizal@123",type,faizal@123,"admin.city_admin.input_password"
+13.Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+14.Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+15. Click on the "Transport Service" → "Auto Ride" checkbox,click,,"admin.city_admin.chk_transport_autoride"
+16.Click on the "Customers" → "Add Customers" checkbox,click,,"admin.city_admin.chk_customer_add"
+17.Click on the "Customers" → "Verified Customers"checkbox,click,,"admin.city_admin.chk_customer_verified"
+18.Click on the "Customers" → "Non Verified Customers" checkbox,click,,"admin.city_admin.chk_customer_unverified"
+19.Click on the "Customers" → "Blocked Customers" checkbox,click,,"admin.city_admin.chk_customer_blocked"
+20.Click on the "Customers" → "Deleted Customers" checkbox,click,,"admin.city_admin.chk_customer_deleted"
+21.Click on the "Providers" → "Transport Providers List" checkbox,click,,"admin.city_admin.chk_provider_list"
+22.Click on the "Drivers" → "Add Driver" checkbox,click,,"admin.city_admin.chk_driver_add"
+23.Click on the "Drivers" → "Approved Drivers" checkbox,click,,"admin.city_admin.chk_driver_approved"
+24.Click on the "Drivers" → "Un-Approved Drivers" checkbox,click,,"admin.city_admin.chk_driver_unapproved"
+25.Click on the "Drivers" → "Blocked Drivers" checkbox,click,,"admin.city_admin.chk_driver_blocked"
+26.Click on the "Drivers" → "Reject Drivers" checkbox,click,,"admin.city_admin.chk_driver_rejected"
+27.Click on the "Drivers" → "Deleted Drivers" checkbox,click,,"admin.city_admin.chk_driver_deleted"
+28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox,click,,"admin.city_admin.chk_subscription_plan"
+29.Click on the "Cash Out" → "Driver Cash Out" checkbox,click,,"admin.city_admin.chk_cashout"
+30.Click on the "Report Issue" → "Customer Report Issues" checkbox,click,,"admin.city_admin.chk_report_customer"
+31.Click on the "Report Issue" → "Driver Report Issues" checkbox,click,,"admin.city_admin.chk_report_driver"
+32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"admin.city_admin.chk_report_provider"
+33.Click on the "Report Issue" → "Report issue settings" checkbox,click,,"admin.city_admin.chk_report_settings"
+34.Click on the "Report Issue" → "FAQs" checkbox,click,,"admin.city_admin.chk_report_faqs"
+35.Click Submit,click,,"web.global.login.submit_btn"
+36. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+37.Filter admin name,type,{adminName},"admin.city_admin.input_name_filter"</t>
+  </si>
+  <si>
+    <t>Test Steps Deleted</t>
+  </si>
+  <si>
+    <t>111.Click Settings ,click,, "admin.transport.menu.settings"
+112.Click Customer Loyalty Settings,click,, "admin.transport.loyalty.menu_item"
+113.Open status Allow Customer loyalty points,click,, "admin.transport.loyalty.status.dropdown"
+114.Open status Allow Customer loyalty points,click,, "admin.transport.loyalty.status.dropdown"
+115.Select ON,click,, "admin.transport.loyalty.status.on_option"
+116.Enter Minimum order amount for eligibility to redeem loyalty points, type, 100, "admin.transport.loyalty.min_redeem.input"
+117.Enter Loyalty points redeem per order (in %) (% of order amount), type, 10, "admin.transport.loyalty.pct_cap.input"
+118.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5, "admin.transport.loyalty.ratio.input"
+119.Click Submit ,click,, "web.global.action.submit"
+120.Wait For Sucess, wait_until_visible, , "web.global.toast.info"</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2. Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+4.Click  Add Category,click,, "admin.transport.add_category.btn"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
+7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
+9.wait,2000,,
+10.Open status Dropdown,click,, "admin.transport.status.dropdown"
+11.Select Activate,click,, "admin.transport.status.activate_option"
+12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
+13.Select {areaName},click,, "admin.transport.city.dynamic_option"
+14.Click  Submit,click,, "web.global.action.submit"
+15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
+16.wait,2000,,
+17.Click  back,click,, "admin.transport.back.btn"
+18. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+19.Click Transports Services Menu,click,, "admin.transport.menu.card"
+20.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+21.Click Home Icon ,click,, "admin.transport.home.icon"
+22.Click Settings ,click,, "admin.transport.menu.settings"
+23.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
+24.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
+26.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
+27.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
+28.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
+29.Select Amount,click,, "admin.transport.status.amount_option"
+30.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
+31.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
+32.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
+33.Select Amount,click,, "admin.transport.status.amount_option"
+34.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
+35.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
+36.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
+37.Select Amount,click,, "admin.transport.status.amount_option"
+38.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
+39.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
+40.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
+41.Select Amount,click,, "admin.transport.status.amount_option"
+42.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
+43.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
+44.Select Amount,click,, "admin.transport.status.amount_option"
+45.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
+46.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
+47.Select Amount,click,, "admin.transport.status.amount_option"
+48.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
+49.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
+50.Select Amount,click,, "admin.transport.status.amount_option"
+51.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
+52.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
+53.Select Amount,click,, "admin.transport.status.amount_option"
+54.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
+55.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
+56.Select Active,click,, "admin.transport.status.active_option"
+57.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
+58.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
+59.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
+60.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
+61.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
+62.Select Active,click,, "admin.transport.status.active_option"
+63.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
+64.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
+65.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
+66.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
+67.Select Amount,click,, "admin.transport.status.amount_option"
+68.Enter  Price, type,50, "admin.transport.night.price.input"
+69.Click  Submit,click,, "web.global.action.submit"
+70.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
+71.Click Settings ,click,, "admin.transport.menu.settings"
+72.Click Promocode,click,, "admin.transport.promo.menu_item"
+73.Click Add Promo Code ,click,, "admin.transport.promo.add.btn"
+74.Open User List Dropdown,click,, "admin.transport.promo.user_list.dropdown"
+75.Select User,click,, "admin.transport.promo.user_option"
+76.Click Code Name Box,click,, "admin.transport.promo.codename.input"
+77.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "admin.transport.promo.codename.input"
+78.Open Discout Type Dropdown,click,, "admin.transport.promo.discount_type.dropdown"
+79.Select Discout Type,click,, "admin.transport.promo.discount_type.amount_option"
+80.Enter Expiry Date,type,12122026, "admin.transport.promo.expiry.input"
+81.Enter Discount Amount, type, 100, "admin.transport.promo.amount.input"
+82.Enter Minimum Order Amount, type, 1000, "admin.transport.promo.min_order.input"
+83.Enter Maximum Discount Amount, type, 100, "admin.transport.promo.max_discount.input"
+84.Enter Coupon Limit, type, 5, "admin.transport.promo.coupon_limit.input"
+85.Enter Usage Limit for One User, type, 2, "admin.transport.promo.user_limit.input"
+86.Enter Promo Code Description, type, Promo Dode For Gold Member, "admin.transport.promo.desc.textarea"
+87.Click Submit ,click,, "web.global.action.submit"
+88.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+89.wait,2000,,
+90.Click Settings ,click,, "admin.transport.menu.settings"
+91.Click Service Settings ,click,, "admin.transport.rules.menu_item"
+92.Enter Driver Accept Timeout, type, 60, "admin.transport.rules.timeout.input"
+93.Enter Driver Serach Radius, type, 50, "admin.transport.rules.radius.input"
+94.Click Submit ,click,, "web.global.action.submit"
+95.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+96.wait,1000,,
+97.Click Settings ,click,, "admin.transport.menu.settings"
+98.Click Requirment Document ,click,, "admin.transport.docs.menu_item"
+99.Click Add Document ,click,, "admin.transport.docs.add.btn"
+100.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "admin.transport.docs.name.input"
+101.Open status Dropdown,click,, "admin.transport.docs.status.dropdown"
+102.Select Active,click,, "admin.transport.status.active_option"
+103.Click Document Expiry ,click,, "admin.transport.docs.expiry.checkbox"
+104.Click Mandatory Document ,click,, "admin.transport.docs.mandatory.checkbox"
+105.Click  Require Proof Number,click,, "admin.transport.docs.proof_no.checkbox"
+106.Enter Display Order, type, 10, "admin.transport.docs.order.input"
+107.Click Submit ,click,, "web.global.action.submit"
+108.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+109.Filter Document List,type,{documentName}, "admin.transport.docs.grid.name_filter"
+110.wait,1000,,
+111. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+112.Click drivers menu,click,, "admin.drivers.menu.icon"
+113.Click Add Driver menu,click,, "admin.drivers.add_menu.link"
+114.Wait For Add Driver, wait_until_visible,, "admin.drivers.add_page.header"
+115.Click Service Category Dropdown,click,, "admin.drivers.service_dropdown.select"
+116.Select Bus Ride Option,click,, "admin.transport.dropdown.dynamic_service"
+117.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "admin.drivers.fullname.input"
+118.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "admin.drivers.email.input"
+119.Enter Contact Number, type, {randomPhone}&gt;&gt;busPhone, "admin.drivers.phone.input"
+120.Click Whatspp,click,, "admin.drivers.whatsapp.checkbox"
+121.Enter Whatspp Number,type,{busPhone}, "admin.drivers.whatsapp_phone.input"
+122.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "admin.drivers.profile_image.file"
+123.Select Source,click,, "admin.drivers.source_dropdown.select"
+124.Select Instagram,click,, "admin.drivers.instagram_option.span"
+125.Select Male Gender, click, , "admin.drivers.male_gender.div"
+126.Click Vehicle Type Dropdown,click,, "admin.drivers.vehicle_dropdown.select"
+127.Select  volvo Option,click,, "admin.transport.dropdown.dynamic_vehicle"
+128.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+129.Enter Plate No, type, KL-01-AB-1634, "admin.drivers.plateno.input"
+130. Enter Model Name, type, deisel, "admin.drivers.modelname.input"
+131.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "admin.drivers.vehicle_image.file"
+132.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+133.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
+134.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+135.Enter Account Holder Name, type, {busDriverName}, "admin.drivers.accountholder.input"
+136.Enter Payment Email Address, type, {busEmail}, "admin.drivers.paymentemail.input"
+137.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+138.Click Submit, click, , "web.global.action.submit"
+139.Wait For Driver Added,wait_until_visible, , "web.global.toast.success"
+140.Wait for Toast to hide, wait, 1000,
+141. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+142.Click drivers menu,click,, "admin.drivers.menu.icon"
+143.Click Pending Documents,click,, "admin.drivers.pending_docs.link"
+144.Filter by Name,type,{busDriverName}, "admin.drivers.name_filter.input"
+145.Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+146.Click Doc Icon,click,, "admin.drivers.docs.icon"
+147.Driver Required Documents,verify,, "admin.drivers.required_docs.header"
+148.FilterDocumet List,type,{documentName}, "admin.drivers.docs_filter.input"
+149.Add Driving License,click,, "admin.drivers.docs.edit_icon"
+150.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+151.Enter Expiry Date,type,12-12-2026, "admin.drivers.doc_expiry.input"
+152.Click Submit, click, , "web.global.action.submit"
+153.Wait For Updated Succesfully, wait_until_visible, , "web.global.toast.updated"
+154.Click Approve Driver,click,, "admin.drivers.docs.approval"
+155.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+156. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+157.Click drivers menu,click,, "admin.drivers.menu.icon"
+158.Click Approved Drivers,click,, "admin.drivers.approved_docs.link"
+159.Wait For Approved Drivers List, wait_until_visible,, "admin.drivers.approved_page.header"
+160.Filter Approved Driver,type,{busDriverName}, "admin.drivers.name_filter.input"
+161.Click Transports Services Icon,click,, "admin.drivers.menu.icon"
+162.Click Transports Services Menu,click,, "admin.transport.menu.card"
+163.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+164.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+165.Click Edit Icon ,click,, "admin.drivers.docs.edit_icon"
+166.wait,2000,,
+167.Scroll Grid, tab, 5, "admin.transport.name.input"
+168.wait,2000,,
+169.Open status Dropdown,click,, "admin.transport.status.dropdown"
+170.Select Deactivate,click,, "admin.transport.status.deactivate_option"
+171.Click  Submit,click,, "web.global.action.submit"
+172.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+173.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -3534,7 +3550,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -3603,13 +3619,13 @@
         <v>27</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -3675,7 +3691,7 @@
         <v>30</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>31</v>
@@ -3747,13 +3763,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -3819,13 +3835,13 @@
         <v>55</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>59</v>
@@ -3891,7 +3907,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
@@ -3963,7 +3979,7 @@
         <v>41</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>57</v>
@@ -4035,13 +4051,13 @@
         <v>71</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>73</v>
@@ -4101,19 +4117,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>66</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>68</v>
@@ -4188,7 +4204,7 @@
         <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>
@@ -4264,7 +4280,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>
@@ -4296,7 +4312,7 @@
     <col min="4" max="4" width="34.77734375" customWidth="1"/>
     <col min="5" max="5" width="64" customWidth="1"/>
     <col min="6" max="6" width="32.6640625" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
+    <col min="7" max="7" width="44.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -4319,7 +4335,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
+        <v>108</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4339,10 +4355,13 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>38</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -4384,7 +4403,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4398,19 +4417,19 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4459,7 +4478,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4473,19 +4492,19 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4534,7 +4553,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4548,19 +4567,19 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4576,7 +4595,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DB4E5D-EBF5-4B6A-BF83-7934D70C5535}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5E7D15-8F85-42A0-A3E4-72E2C74068F3}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4586,7 +4605,7 @@
     <col min="4" max="4" width="34.109375" customWidth="1"/>
     <col min="5" max="5" width="69.33203125" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="61.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -4609,7 +4628,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
+        <v>111</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4623,16 +4642,19 @@
         <v>61</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>64</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>63</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4690,22 +4712,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
76th Commit: Locator Migration Completed
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC13A97E-358D-43E7-AB26-196297D4DAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2782A3-6539-4CC8-BB61-AFA4B194CB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -26,9 +26,9 @@
     <sheet name="StoreOperations" sheetId="42" r:id="rId11"/>
     <sheet name="StoreStatusManagement" sheetId="43" r:id="rId12"/>
     <sheet name="DeliveryServiceCompleteTest" sheetId="44" r:id="rId13"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId14"/>
-    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId15"/>
-    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId16"/>
+    <sheet name="AddProvider" sheetId="45" r:id="rId14"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="46" r:id="rId15"/>
+    <sheet name="SubscriptionPlanTest" sheetId="47" r:id="rId16"/>
     <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId17"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -898,111 +898,6 @@
     <t>Validate the end-to-end creation of a Customer.</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'ON-DEMAND SERVICES')]"
-4.Filter service List,type,Plumbers,"//input[@aria-label='Services Filter Input']"
-5.Click Home Icon Plumbers,click,,"//div[@role='row'][.//span[text()='Plumbers']]//i[@title='Home']"
-6.Verify Plumbers Summary,verify,,"//div[contains(text(),'Plumbers Summary')]"
-7.Click  Providers,click,,"//button[contains(., 'Providers')]"
-8.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-9.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "//input[@placeholder='Provider Full Name']"
-11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "//input[@type='file']"
-12.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "//input[@placeholder='Unique Email']"
-13.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-14.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-15.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-16.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-17.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-18.Enter Provider Address, type, plumber chennai, "//input[@placeholder='Enter provider Address']"
-19.wait,1000,,
-20.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-21.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-22.wait,1000,,
-23.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-24.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-25.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-26.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-27.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-28.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-29.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-30.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-31.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-32.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-33.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-34.Enter Accont Holder Name, type, {plumberName}, "//input[@placeholder='Account Holder Name']"
-35.Enter Payment Email Address, type, {plumberEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-36.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-37.Click Save, click, , "//button[@type='submit']"
-38.Verify Sucess, verify, , "//div[@aria-label='Info']"
-39.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-40.Click  Providers,click,,"//button[contains(., 'Providers')]"
-41.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-42.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-43.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-44. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
-45.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-46.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-47.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-48.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-49.Click Submit, click, , "//button[normalize-space()='Submit']"
-50.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-51.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-52.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-53.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-54.Click Back, click, , "//button[@class='buttonWidget']"
-55.Click  Providers,click,,"//button[contains(., 'Providers')]"
-56.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-57.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
-58.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-59.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-60.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-61.Click Back, click, , "//button[@class='buttonWidget']"
-62.Verify Approved Provider,verify,,"//div[normalize-space()='Approved Plumbers Service Providers']"
-63.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-64.Scroll Grid, tab, 11, "//input[@aria-label='Provider Name Filter Input']"
-65.Click Wallet Icon,click,,"//i[@class='bi bi-cash-stack cursor-pointer gridIcon Navigate']"
-66.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-67.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-68.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-69.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-70.Click Submit, click, , "//button[normalize-space()='Submit']"
-71.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-72.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-73.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-74.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-75.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-76.Click Submit, click, , "//button[normalize-space()='Submit']"
-77.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-78.Click Back, click, , "//button[normalize-space()='Back']"
-79.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-80.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-81.FilterDocumet List,type,Store Address,"//input[@aria-label='Document Name Filter Input']"
-82.Click Reject Document,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-83.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-84.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-85..Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-86.Click Back, click, , "//button[@class='buttonWidget']"
-87.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-88.Scroll Grid, tab, 13, "//input[@aria-label='Provider Name Filter Input']"
-89.Click Block Provider,click,,"//i[@title='Block Provider']"
-90.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-91. Blocking Reason,type,customer complaints,"//textarea[@id='swal2-textarea']"
-92.Click block  Yes,click,,"//button[normalize-space()='Yes']"
-93.Click  Providers,click,,"//button[contains(., 'Providers')]"
-94.Select Blocked Providers,click,,"//div[contains(text(), 'Blocked Providers')]"
-95.Verify Blocked Provider,verify,,"//div[normalize-space()='Blocked Plumbers Service Providers']"
-96.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-97.Scroll Grid, tab, 12, "//input[@aria-label='Provider Name Filter Input']"
-98.Click Unblock Provider,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-99.Click  Providers,click,,"//button[contains(., 'Providers')]"
-100.Select Provider List,click,,"//div[contains(text(), 'Provider List')]"
-101.Filter Plumber List,type,{plumberName},"//input[@aria-label='Provider Name Filter Input']"
-102.wait,1000,,
-</t>
-  </si>
-  <si>
     <t>Add New Delivery Service &amp;  Category</t>
   </si>
   <si>
@@ -1381,150 +1276,6 @@
     </r>
   </si>
   <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-2.Click Provider Services,click,,"//h2[contains(text(), 'Provider Services')]"
-3.Verify Provider Services,verify,,"//div[normalize-space()='ON-DEMAND SERVICES']"
-4.Click  Add New Services,click,,"//button[normalize-space()='Add New Services']"
-5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "//input[@placeholder='Service Name']"
-6.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-7.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-8.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-9.Enter Slug, type, painter, "//input[@placeholder='Slug']"
-10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-11.wait,2000,,
-12.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-13.Select Activate,click,,"//li[@aria-label='Activate']"
-14.Open Select City Dropdown,click,,"//div[contains(@class, 'p-multiselect-label-container')]"
-15.Select {areaName},click,,"//li[contains(@aria-label, '{areaName}')]"
-16.Click  Submit,click,,"//button[normalize-space()='Submit']"
-17.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click Settings ,click,,"//button[contains(., 'Settings')]"
-20.Click Requirment Document ,click,,"//div[normalize-space()='Required Document']"
-21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, documet{randomAlpha}&gt;&gt; providerDocumentName, "//input[@placeholder='Type here']"
-23.Open status Dropdown,click,,"//span[@aria-label='Status']"
-24.Select Active,click,,"//li[@aria-label='Active']"
-25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-26.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-27.Click Submit ,click,,"//button[normalize-space()='Submit']"
-28.Verify Sucess, verify, , "//div[@aria-label='Info']"
-29.Filter Document List,type,{providerDocumentName},"//input[@aria-label='Name Filter Input']"
-30.Click Settings ,click,,"//button[contains(., 'Settings')]"
-31.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
-32.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-33.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-34.Select User,click,,"//li[@aria-label='{customerName}']"
-35.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-35.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; providerPromoCodeName, "//input[@placeholder='Code Name']"
-36.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-37.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-38.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-39.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-40.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-41.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-42.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-43.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-44.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-45.Click Submit ,click,,"//button[normalize-space()='Submit']"
-46.Verify Sucess, verify, , "//div[@aria-label='Info']"
-47.Filter PromoCode List,type,{providerPromoCodeName},"//input[@aria-label='Promocode Filter Input']"
-48.Click  Providers,click,,"//button[contains(., 'Providers')]"
-49.Select Add Providers,click,,"//div[contains(text(), 'Add Providers')]"
-50.Verify Add Provider,verify,,"//h1[text()=' Add Provider ']"
-51.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "//input[@placeholder='Provider Full Name']"
-52.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file']"
-53.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "//input[@placeholder='Unique Email']"
-54.Enter Contact Number, type, {randomPhone}, "//input[@placeholder='Unique Contact Number']"
-55.Enter Landmark, type, Near LIC Building, "//input[@placeholder='Provider Landmark']"
-56.Open Delivery Radius Dropdown,click,,"//select[@formcontrolname='serviceRadius']"
-57.Select Twenty Five Kilometer,click,,"//option[text()='25 KM']"
-58.Enter Minimum Order, type, 10, "//input[@placeholder='Minimum Order']"
-59.Enter Provider Address, type, painter chennai, "//input[@placeholder='Enter provider Address']"
-60.wait,1000,,
-61.Select First Option,arrow_down,,"//input[@placeholder='Enter provider Address']"
-62.Confirm Option,press_enter,,"//input[@placeholder='Enter provider Address']"
-63.wait,1000,,
-64.Click Everyday Checkbox, click, , "//span[text()='EveryDay']/preceding-sibling::input"
-65.Click 09:00 AM-10:00 AM, click, , "//button[normalize-space()='09:00 AM-10:00 AM']"
-66.Click 10:00 AM-11:00 AM, click, , "//button[normalize-space()='10:00 AM-11:00 AM']"
-67.Click 11:00 AM-12:00 PM, click, , "//button[normalize-space()='11:00 AM-12:00 PM']"
-68.Click 12:00 PM-01:00 PM, click, , "//button[normalize-space()='12:00 PM-01:00 PM']"
-69.Click 02:00 PM-03:00 PM, click, , "//button[normalize-space()='02:00 PM-03:00 PM']"
-70.Click 03:00 PM-04:00 PM, click, , "//button[normalize-space()='03:00 PM-04:00 PM']"
-71.Enter Bank Name, type, federal, "//input[@placeholder='Bank Name']"
-72.Enter Bank Location,type, chennai, "//input[@placeholder='Bank Location(City Name)']"
-73.Scroll Grid, tab, 1, "//input[@placeholder='Bank Location(City Name)']"
-74.Enter Account Number, type, 123456789012, "//input[@placeholder='Account Number']"
-75.Enter Accont Holder Name, type, {painterName}, "//input[@placeholder='Account Holder Name']"
-76.Enter Payment Email Address, type, {painterEmail}, "//input[@placeholder='Email Address for Payment Notification']"
-77.Enter BIC Code, type, 1234, "//input[@placeholder='BIC Code']"
-78.Click Save, click, , "//button[@type='submit']"
-79.Verify Sucess, verify, , "//div[@aria-label='Info']"
-80.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-81.Click  Providers,click,,"//button[contains(., 'Providers')]"
-82.Select Pending Document Providers,click,,"//div[normalize-space()='Pending Document Providers']"
-83.Filter Plumber List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-84.Click Document Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-85. Provider Required Documents,verify,,"//div[contains(text(),'Documents')]"
-86.FilterDocumet List,type,{providerDocumentName},"//input[@aria-label='Document Name Filter Input']"
-87.Add Address Proof,click,,"(//i[contains(@class, 'Edit')])[1]"
-88.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-89.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-90.Click Submit, click, , "//button[normalize-space()='Submit']"
-91.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-92.FilterDocumet List,type,{providerDocumentName},"//input[@aria-label='Document Name Filter Input']"
-93.Click Approve Store,click,,"//div[@row-index='0']//i[contains(@class, 'bi-hand-thumbs-up-fill')]"
-94.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-95.Click Back, click, , "//button[@class='buttonWidget']"
-96.Click  Providers,click,,"//button[normalize-space()='Category']"
-97.Click  Add New Category,click,,"//button[normalize-space()='ADD CATEGORY']"
-98.Enter Category Name, type,residentialPainter{randomAlpha}&gt;&gt; painterCategoryName, "//input[@placeholder='Enter the category name']"
-99.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "//input[@placeholder='Category Name (in Tamil)']"
-100.Enter Category Name Arabic, type, دهان سكني, "//input[@placeholder='Category Name (in Arabic)']"
-101.Enter Category Name Hindi, type, आवासीय पेंटर, "//input[@placeholder='Category Name (in Hindi)']"
-102.Open Category status Dropdown,click,,"//span[@aria-label='Select a category status']"
-103.Select Activate,click,,"//li[@aria-label='Active']"
-104.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "//input[@type='file' and @accept='image/*']"
-105.wait,2000,,
-106.Click  Submit,click,,"//button[normalize-space()='Submit']"
-107.Filter Category Name,type,{painterCategoryName},"//input[@aria-label='Category Name Filter Input']"
-108.Click  Providers,click,,"//button[contains(., 'Providers')]"
-109.Select Provider List,click,,"//div[normalize-space()='Provider List']"
-110.Filter Painter List,type,{painterName},"//input[@aria-label='Provider Name Filter Input']"
-111.Scroll Grid, tab, 7, "//input[@aria-label='Provider Name Filter Input']"
-112.Click Package Icon,click,,"//i[@class='bi bi-box-seam cursor-pointer gridIcon Navigate']"
-113.Click  Add Package,click,,"//button[normalize-space()='Add Package']"
-114.Open Category  Dropdown,click,,"//span[@aria-label='Package Category']"
-115.Select Activate,click,,"//li[@aria-label='{painterCategoryName}']"
-116.Enter Package Name, type, package{randomAlpha}&gt;&gt; packageName, "//input[@placeholder='Package Name']"
-117.Enter Amount, type, 1000, "//input[@placeholder='Amount Value']"
-118.Open Max Book Quantity  Dropdown,click,,"//span[@aria-label='Package Max Book Quantity']"
-119.Select 4,click,,"//li[@aria-label='4']"
-120.Open Status Dropdown,click,,"//span[@aria-label='select Status']"
-121.Select Activate,click,,"//li[@aria-label='Activate']"
-122.Enter Description, type, Premium residential painting package, "//textarea[@placeholder='Description']"
-123.Click  Submit,click,,"//button[normalize-space()='Submit']"
-124.wait,1000,,
-125.Click  back,click,,"//button[normalize-space()='Back']"
-126.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-127.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-128.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-129.Click Edit Icon ,click,,"//i[@title='Edit']"
-130.Enter Service Name Tamil, type, பெயிண்டர், "//input[@placeholder='Service Name (in Tamil)']"
-131.Enter Service Name Arabic, type, دهان, "//input[@placeholder='Service Name (in Arabic)']"
-132.Enter Service Name Hindi, type, पेंटर, "//input[@placeholder='Service Name (in Hindi)']"
-133.Scroll Grid, tab, 4, "//input[@placeholder='Service Name (in Hindi)']"
-134.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-135.Select Deactivate,click,,"//li[@aria-label='Deactivate']"
-136.Click  Submit,click,,"//button[normalize-space()='Submit']"
-137.Click  back,click,,"//button[normalize-space()='Back']"
-138.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
-139.Click Delivery Services,click,,"//h2[contains(text(), 'Provider Services')]"
-140.Filter Services List,type,{serviceName},"//input[@aria-label='Services Filter Input']"
-141.wait,1000,,</t>
-  </si>
-  <si>
     <t>Add New  Store, Provider , Driver &amp;  Customer Subscription Plan</t>
   </si>
   <si>
@@ -1603,131 +1354,6 @@
   </si>
   <si>
     <t>Super Admin Login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-3.Click Store subscription plan,click,,"//span[normalize-space()='Store Subscription Plan']"
-4.Verify Store Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Store']"
-5.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-7.Select Food Delivery,click,,"//li[@aria-label='Food Delivery']"
-8.Enter Store Plan Name, type, StorePlan{randomAlpha}&gt;&gt; storeSubscriptionName, "//input[@placeholder='Plan Name']"
-9.Enter Store Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-10.Enter Store Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-11.Enter Store Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-12.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-13.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-14.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-15.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-16.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-17.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-18.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-19.Select On,click,,"//li[@aria-label='on']"
-20.Click Submit ,click,,"//button[normalize-space()='Submit']"
-21.Filter Services List,type,{storeSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-22.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-23.Click Close ,click,,"//button[normalize-space()='Close']"
-24.Click Active ,click,,"//i[@title='Active']"
-25.wait,2000,,
-26.Click Deactive,click,,"//i[@title='Inactive']"
-27.wait,2000,,
-28.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-29.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-30.wait,3000,,
-31.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-32.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-33.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
-34.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
-35.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
-36.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-37.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
-38.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
-39.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-40.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
-41.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
-42.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
-43.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
-44.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-45.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-46.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
-47.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
-48.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
-49.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-50.Select On,click,,"//li[@aria-label='on']"
-51.Click Submit ,click,,"//button[normalize-space()='Submit']"
-52.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-53.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-54.Click Close ,click,,"//button[normalize-space()='Close']"
-55.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-56.wait,2000,,
-57.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-58.wait,2000,,
-59.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-60.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-61.wait,3000,,
-62.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-63.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-64.Click Provider subscription plan,click,,"//span[normalize-space()='Provider Subscription Plan']"
-65.Verify Provider Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Provider']"
-66.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-67.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-68.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-69.Enter Provider Plan Name, type, ProviderPlan{randomAlpha}&gt;&gt; providerSubscriptionName, "//input[@placeholder='Plan Name']"
-70.Enter Provider Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic):']"
-71.Enter Provider Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-72.Enter Provider Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-73.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-74.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price ']"
-75.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Enter Description(in English):']"
-76.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Enter Description(in Arabic):']"
-77.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Enter Description(in Tamil)']"
-78.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Enter Description(in Hindi']"
-79.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-80.Select On,click,,"//li[@aria-label='on']"
-81.Click Submit ,click,,"//button[normalize-space()='Submit']"
-82.Filter Services List,type,{providerSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-83.Click Edit ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-84.Click Close ,click,,"//button[normalize-space()='Close']"
-85.Click Active ,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-86.wait,2000,,
-87.Click Deactive,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-88.wait,2000,,
-89.Click Delete Plan,click,,"//i[@class='bi bi-trash cursor-pointer gridIcon Delete']"
-90.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-91.wait,3000,,
-92.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-93.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-94.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
-95.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
-96.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-97.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-98.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-99.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
-100.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-101.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-102.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-103.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-104.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
-105.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-106.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-107.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-108.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-109.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-110.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-111.Select On,click,,"//li[@aria-label='on']"
-112.Click Submit ,click,,"//button[normalize-space()='Submit']"
-113.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-114.Click Edit ,click,,"//i[@title='Edit Plan']"
-115.Click Close ,click,,"//button[normalize-space()='Close']"
-116.Click Active ,click,,"//i[@title='Activate Plan']"
-117.wait,2000,,
-118.Click Deactive,click,,"//i[@title='Deactivate Plan']"
-119.wait,2000,,
-120.Click Delete Plan,click,,"//i[@title='Delete Plan']"
-121.Click Confirm Delete,click,,"//button[normalize-space()='Yes, delete it!']"
-122.wait,3000,,
-</t>
   </si>
   <si>
     <t>SA_TS_16</t>
@@ -1998,181 +1624,6 @@
 118.Enter Loyalty points per default currency (for ex. $1 = 10 points), type, 5, "admin.transport.loyalty.ratio.input"
 119.Click Submit ,click,, "web.global.action.submit"
 120.Wait For Sucess, wait_until_visible, , "web.global.toast.info"</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
-2. Click Transports Services Menu,click,, "admin.transport.menu.card"
-3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
-4.Click  Add Category,click,, "admin.transport.add_category.btn"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
-7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
-9.wait,2000,,
-10.Open status Dropdown,click,, "admin.transport.status.dropdown"
-11.Select Activate,click,, "admin.transport.status.activate_option"
-12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
-13.Select {areaName},click,, "admin.transport.city.dynamic_option"
-14.Click  Submit,click,, "web.global.action.submit"
-15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
-16.wait,2000,,
-17.Click  back,click,, "admin.transport.back.btn"
-18. Click Dashboard Icon,click,, "web.global.menu.dashboard"
-19.Click Transports Services Menu,click,, "admin.transport.menu.card"
-20.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
-21.Click Home Icon ,click,, "admin.transport.home.icon"
-22.Click Settings ,click,, "admin.transport.menu.settings"
-23.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
-24.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
-25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
-26.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
-27.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
-28.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
-29.Select Amount,click,, "admin.transport.status.amount_option"
-30.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
-31.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
-32.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
-33.Select Amount,click,, "admin.transport.status.amount_option"
-34.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
-35.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
-36.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
-37.Select Amount,click,, "admin.transport.status.amount_option"
-38.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
-39.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
-40.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
-41.Select Amount,click,, "admin.transport.status.amount_option"
-42.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
-43.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
-44.Select Amount,click,, "admin.transport.status.amount_option"
-45.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
-46.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
-47.Select Amount,click,, "admin.transport.status.amount_option"
-48.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
-49.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
-50.Select Amount,click,, "admin.transport.status.amount_option"
-51.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
-52.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
-53.Select Amount,click,, "admin.transport.status.amount_option"
-54.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
-55.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
-56.Select Active,click,, "admin.transport.status.active_option"
-57.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
-58.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
-59.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
-60.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
-61.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
-62.Select Active,click,, "admin.transport.status.active_option"
-63.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
-64.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
-65.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
-66.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
-67.Select Amount,click,, "admin.transport.status.amount_option"
-68.Enter  Price, type,50, "admin.transport.night.price.input"
-69.Click  Submit,click,, "web.global.action.submit"
-70.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
-71.Click Settings ,click,, "admin.transport.menu.settings"
-72.Click Promocode,click,, "admin.transport.promo.menu_item"
-73.Click Add Promo Code ,click,, "admin.transport.promo.add.btn"
-74.Open User List Dropdown,click,, "admin.transport.promo.user_list.dropdown"
-75.Select User,click,, "admin.transport.promo.user_option"
-76.Click Code Name Box,click,, "admin.transport.promo.codename.input"
-77.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "admin.transport.promo.codename.input"
-78.Open Discout Type Dropdown,click,, "admin.transport.promo.discount_type.dropdown"
-79.Select Discout Type,click,, "admin.transport.promo.discount_type.amount_option"
-80.Enter Expiry Date,type,12122026, "admin.transport.promo.expiry.input"
-81.Enter Discount Amount, type, 100, "admin.transport.promo.amount.input"
-82.Enter Minimum Order Amount, type, 1000, "admin.transport.promo.min_order.input"
-83.Enter Maximum Discount Amount, type, 100, "admin.transport.promo.max_discount.input"
-84.Enter Coupon Limit, type, 5, "admin.transport.promo.coupon_limit.input"
-85.Enter Usage Limit for One User, type, 2, "admin.transport.promo.user_limit.input"
-86.Enter Promo Code Description, type, Promo Dode For Gold Member, "admin.transport.promo.desc.textarea"
-87.Click Submit ,click,, "web.global.action.submit"
-88.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-89.wait,2000,,
-90.Click Settings ,click,, "admin.transport.menu.settings"
-91.Click Service Settings ,click,, "admin.transport.rules.menu_item"
-92.Enter Driver Accept Timeout, type, 60, "admin.transport.rules.timeout.input"
-93.Enter Driver Serach Radius, type, 50, "admin.transport.rules.radius.input"
-94.Click Submit ,click,, "web.global.action.submit"
-95.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-96.wait,1000,,
-97.Click Settings ,click,, "admin.transport.menu.settings"
-98.Click Requirment Document ,click,, "admin.transport.docs.menu_item"
-99.Click Add Document ,click,, "admin.transport.docs.add.btn"
-100.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "admin.transport.docs.name.input"
-101.Open status Dropdown,click,, "admin.transport.docs.status.dropdown"
-102.Select Active,click,, "admin.transport.status.active_option"
-103.Click Document Expiry ,click,, "admin.transport.docs.expiry.checkbox"
-104.Click Mandatory Document ,click,, "admin.transport.docs.mandatory.checkbox"
-105.Click  Require Proof Number,click,, "admin.transport.docs.proof_no.checkbox"
-106.Enter Display Order, type, 10, "admin.transport.docs.order.input"
-107.Click Submit ,click,, "web.global.action.submit"
-108.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-109.Filter Document List,type,{documentName}, "admin.transport.docs.grid.name_filter"
-110.wait,1000,,
-111. Click Dashboard Icon,click,, "web.global.menu.dashboard"
-112.Click drivers menu,click,, "admin.drivers.menu.icon"
-113.Click Add Driver menu,click,, "admin.drivers.add_menu.link"
-114.Wait For Add Driver, wait_until_visible,, "admin.drivers.add_page.header"
-115.Click Service Category Dropdown,click,, "admin.drivers.service_dropdown.select"
-116.Select Bus Ride Option,click,, "admin.transport.dropdown.dynamic_service"
-117.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "admin.drivers.fullname.input"
-118.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "admin.drivers.email.input"
-119.Enter Contact Number, type, {randomPhone}&gt;&gt;busPhone, "admin.drivers.phone.input"
-120.Click Whatspp,click,, "admin.drivers.whatsapp.checkbox"
-121.Enter Whatspp Number,type,{busPhone}, "admin.drivers.whatsapp_phone.input"
-122.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "admin.drivers.profile_image.file"
-123.Select Source,click,, "admin.drivers.source_dropdown.select"
-124.Select Instagram,click,, "admin.drivers.instagram_option.span"
-125.Select Male Gender, click, , "admin.drivers.male_gender.div"
-126.Click Vehicle Type Dropdown,click,, "admin.drivers.vehicle_dropdown.select"
-127.Select  volvo Option,click,, "admin.transport.dropdown.dynamic_vehicle"
-128.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
-129.Enter Plate No, type, KL-01-AB-1634, "admin.drivers.plateno.input"
-130. Enter Model Name, type, deisel, "admin.drivers.modelname.input"
-131.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "admin.drivers.vehicle_image.file"
-132.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
-133.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
-134.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
-135.Enter Account Holder Name, type, {busDriverName}, "admin.drivers.accountholder.input"
-136.Enter Payment Email Address, type, {busEmail}, "admin.drivers.paymentemail.input"
-137.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
-138.Click Submit, click, , "web.global.action.submit"
-139.Wait For Driver Added,wait_until_visible, , "web.global.toast.success"
-140.Wait for Toast to hide, wait, 1000,
-141. Click Dashboard Icon,click,, "web.global.menu.dashboard"
-142.Click drivers menu,click,, "admin.drivers.menu.icon"
-143.Click Pending Documents,click,, "admin.drivers.pending_docs.link"
-144.Filter by Name,type,{busDriverName}, "admin.drivers.name_filter.input"
-145.Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
-146.Click Doc Icon,click,, "admin.drivers.docs.icon"
-147.Driver Required Documents,verify,, "admin.drivers.required_docs.header"
-148.FilterDocumet List,type,{documentName}, "admin.drivers.docs_filter.input"
-149.Add Driving License,click,, "admin.drivers.docs.edit_icon"
-150.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
-151.Enter Expiry Date,type,12-12-2026, "admin.drivers.doc_expiry.input"
-152.Click Submit, click, , "web.global.action.submit"
-153.Wait For Updated Succesfully, wait_until_visible, , "web.global.toast.updated"
-154.Click Approve Driver,click,, "admin.drivers.docs.approval"
-155.Verify Updated Succesfully, verify, , "web.global.toast.updated"
-156. Click Dashboard Icon,click,, "web.global.menu.dashboard"
-157.Click drivers menu,click,, "admin.drivers.menu.icon"
-158.Click Approved Drivers,click,, "admin.drivers.approved_docs.link"
-159.Wait For Approved Drivers List, wait_until_visible,, "admin.drivers.approved_page.header"
-160.Filter Approved Driver,type,{busDriverName}, "admin.drivers.name_filter.input"
-161.Click Transports Services Icon,click,, "admin.drivers.menu.icon"
-162.Click Transports Services Menu,click,, "admin.transport.menu.card"
-163.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
-164.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
-165.Click Edit Icon ,click,, "admin.drivers.docs.edit_icon"
-166.wait,2000,,
-167.Scroll Grid, tab, 5, "admin.transport.name.input"
-168.wait,2000,,
-169.Open status Dropdown,click,, "admin.transport.status.dropdown"
-170.Select Deactivate,click,, "admin.transport.status.deactivate_option"
-171.Click  Submit,click,, "web.global.action.submit"
-172.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-173.wait,2000,,</t>
   </si>
   <si>
     <t>1.Click Dashboard Icon,click,,"web.global.menu.dashboard"
@@ -2921,7 +2372,306 @@
 53.wait, 2000, , ""</t>
   </si>
   <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+    <t>1.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2.Click Subscription Plan,click,,"admin.subscription.menu_link"
+3.Click Store subscription plan,click,,"admin.subscription.store.tab"
+4.Verify Store Subscription Plan Lists ,verify,,"admin.subscription.store.header"
+5.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+6.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+7.Select Food Delivery,click,,"admin.subscription.common.category.option_food"
+8.Enter Store Plan Name, type, StorePlan{randomAlpha}&gt;&gt; storeSubscriptionName, "admin.subscription.common.name.input"
+9.Enter Store Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+10.Enter Store Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+11.Enter Store Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+12.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+13.Enter Price, type,5000, "admin.subscription.common.price.input"
+14.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.store.desc_english.textarea"
+15.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.store.desc_arabic.textarea"
+16.Enter Plan Description Tamil, type,இட்து விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.store.desc_tamil.textarea"
+17.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.store.desc_hindi.textarea"
+18.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+19.Select On,click,,"admin.subscription.common.status.option_on"
+20.Click Submit ,click,,"web.global.action.submit"
+21.Filter Services List,type,{storeSubscriptionName},"admin.subscription.common.filter.input"
+22.Click Edit ,click,,"admin.subscription.store.edit.icon"
+23.Click Close ,click,,"web.global.action.close"
+24.Click Active ,click,,"admin.subscription.store.active.icon"
+25.wait,2000,,
+26.Click Deactive,click,,"admin.subscription.store.inactive.icon"
+27.wait,2000,,
+28.Click Delete Plan,click,,"admin.subscription.store.delete.icon"
+29.Click Confirm Delete,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+30.wait,3000,,
+31.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+32.Click Subscription Plan,click,,"admin.subscription.menu_link"
+33.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+34.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+35.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+36.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+37.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+38.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+39.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+40.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+41.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+42.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+43.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+44.Enter Price, type,5000, "admin.subscription.common.price.input"
+45.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+46.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+47.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரीமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+48.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+49.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+50.Select On,click,,"admin.subscription.common.status.option_on"
+51.Click Submit ,click,,"web.global.action.submit"
+52.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+53.Click Edit ,click,,"admin.subscription.driver.edit.icon"
+54.Click Close ,click,,"web.global.action.close"
+55.Click Active ,click,,"admin.subscription.driver.active.icon"
+56.wait,2000,,
+57.Click Deactive,click,,"admin.subscription.driver.inactive.icon"
+58.wait,2000,,
+59.Click Delete Plan,click,,"admin.subscription.driver.delete.icon"
+60.Click Confirm Delete,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+61.wait,3000,,
+62. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+63.Click Subscription Plan,click,,"admin.subscription.menu_link"
+64.Click Provider subscription plan,click,,"admin.subscription.provider.tab"
+65.Verify Provider Subscription Plan Lists ,verify,,"admin.subscription.provider.header"
+66.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+67.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+68.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
+69.Enter Provider Plan Name, type, ProviderPlan{randomAlpha}&gt;&gt; providerSubscriptionName, "admin.subscription.common.name.input"
+70.Enter Provider Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.alt_input"
+71.Enter Provider Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+72.Enter Provider Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+73.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+74.Enter Price, type,5000, "admin.subscription.common.price.alt_input"
+75.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.provider.desc_english.textarea"
+76.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.provider.desc_arabic.textarea"
+77.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் सலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.provider.desc_tamil.textarea"
+78.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.provider.desc_hindi.textarea"
+79.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+80.Select On,click,,"admin.subscription.common.status.option_on"
+81.Click Submit ,click,,"web.global.action.submit"
+82.Filter Services List,type,{providerSubscriptionName},"admin.subscription.common.filter.input"
+83.Click Edit ,click,,"admin.subscription.provider.edit.icon"
+84.Click Close ,click,,"web.global.action.close"
+85.Click Active ,click,,"admin.subscription.provider.active.icon"
+86.wait,2000,,
+87.Click Deactive,click,,"admin.subscription.provider.inactive.icon"
+88.wait,2000,,
+89.Click Delete Plan,click,,"admin.subscription.provider.delete.icon"
+90.Click Confirm Delete,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+91.wait,3000,,
+92.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+93.Click Subscription Plan,click,,"admin.subscription.menu_link"
+94.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+95.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+96.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+97.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+98.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
+99.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "admin.subscription.common.name.input"
+100.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+101.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+102.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+103.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+104.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+105.Enter Price, type,5000, "admin.subscription.common.price.input"
+106.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+107.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+108.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+109.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+110.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+111.Select On,click,,"admin.subscription.common.status.option_on"
+112.Click Submit ,click,,"web.global.action.submit"
+113.Filter Services List,type,{custometSubscriptionName},"admin.subscription.common.filter.input"
+114.Click Edit ,click,,"admin.subscription.customer.edit.icon"
+115.Click Close ,click,,"web.global.action.close"
+116.Click Active ,click,,"admin.subscription.customer.active.icon"
+117.wait,2000,,
+118.Click Deactive,click,,"admin.subscription.customer.inactive.icon"
+119.wait,2000,,
+120.Click Delete Plan,click,,"admin.subscription.customer.delete.icon"
+121.Click Confirm Delete,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+122.wait,3000,,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2. Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+4.Click  Add Category,click,, "admin.transport.add_category.btn"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
+7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
+9.wait,2000,,
+10.Open status Dropdown,click,, "admin.transport.status.dropdown"
+11.Select Activate,click,, "admin.transport.status.activate_option"
+12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
+13.Select {areaName},click,, "admin.transport.city.dynamic_option"
+14.Click  Submit,click,, "web.global.action.submit"
+15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
+16.wait,2000,,
+17.Click  back,click,, "admin.transport.back.btn"
+18. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+19.Click Transports Services Menu,click,, "admin.transport.menu.card"
+20.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+21.Click Home Icon ,click,, "admin.transport.home.icon"
+22.Click Settings ,click,, "admin.transport.menu.settings"
+23.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
+24.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
+25.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
+26.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
+27.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
+28.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
+29.Select Amount,click,, "admin.transport.status.amount_option"
+30.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
+31.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
+32.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
+33.Select Amount,click,, "admin.transport.status.amount_option"
+34.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
+35.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
+36.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
+37.Select Amount,click,, "admin.transport.status.amount_option"
+38.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
+39.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
+40.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
+41.Select Amount,click,, "admin.transport.status.amount_option"
+42.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
+43.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
+44.Select Amount,click,, "admin.transport.status.amount_option"
+45.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
+46.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
+47.Select Amount,click,, "admin.transport.status.amount_option"
+48.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
+49.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
+50.Select Amount,click,, "admin.transport.status.amount_option"
+51.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
+52.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
+53.Select Amount,click,, "admin.transport.status.amount_option"
+54.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
+55.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
+56.Select Active,click,, "admin.transport.status.active_option"
+57.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
+58.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
+59.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
+60.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
+61.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
+62.Select Active,click,, "admin.transport.status.active_option"
+63.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
+64.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
+65.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
+66.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
+67.Select Amount,click,, "admin.transport.status.amount_option"
+68.Enter  Price, type,50, "admin.transport.night.price.input"
+69.Click  Submit,click,, "web.global.action.submit"
+70.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
+71.Click Settings ,click,, "admin.transport.menu.settings"
+72.Click Promocode,click,, "admin.transport.promo.menu_item"
+73.Click Add Promo Code ,click,, "admin.transport.promo.add.btn"
+74.Open User List Dropdown,click,, "admin.transport.promo.user_list.dropdown"
+75.Select User,click,, "admin.transport.promo.user_option"
+76.Click Code Name Box,click,, "admin.transport.promo.codename.input"
+77.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; promoCodeName, "admin.transport.promo.codename.input"
+78.Open Discout Type Dropdown,click,, "admin.transport.promo.discount_type.dropdown"
+79.Select Discout Type,click,, "admin.transport.promo.discount_type.amount_option"
+80.Enter Expiry Date,type,12122026, "admin.transport.promo.expiry.input"
+81.Enter Discount Amount, type, 100, "admin.transport.promo.amount.input"
+82.Enter Minimum Order Amount, type, 1000, "admin.transport.promo.min_order.input"
+83.Enter Maximum Discount Amount, type, 100, "admin.transport.promo.max_discount.input"
+84.Enter Coupon Limit, type, 5, "admin.transport.promo.coupon_limit.input"
+85.Enter Usage Limit for One User, type, 2, "admin.transport.promo.user_limit.input"
+86.Enter Promo Code Description, type, Promo Dode For Gold Member, "admin.transport.promo.desc.textarea"
+87.Click Submit ,click,, "web.global.action.submit"
+88.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+89.wait,2000,,
+90.Click Settings ,click,, "admin.transport.menu.settings"
+91.Click Service Settings ,click,, "admin.transport.rules.menu_item"
+92.Enter Driver Accept Timeout, type, 60, "admin.transport.rules.timeout.input"
+93.Enter Driver Serach Radius, type, 50, "admin.transport.rules.radius.input"
+94.Click Submit ,click,, "web.global.action.submit"
+95.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+96.wait,1000,,
+97.Click Settings ,click,, "admin.transport.menu.settings"
+98.Click Requirment Document ,click,, "admin.transport.docs.menu_item"
+99.Click Add Document ,click,, "admin.transport.docs.add.btn"
+100.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "admin.transport.docs.name.input"
+101.Open status Dropdown,click,, "admin.transport.docs.status.dropdown"
+102.Select Active,click,, "admin.transport.status.active_option"
+103.Click Document Expiry ,click,, "admin.transport.docs.expiry.checkbox"
+104.Click Mandatory Document ,click,, "admin.transport.docs.mandatory.checkbox"
+105.Click  Require Proof Number,click,, "admin.transport.docs.proof_no.checkbox"
+106.Enter Display Order, type, 10, "admin.transport.docs.order.input"
+107.Click Submit ,click,, "web.global.action.submit"
+108.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+109.Filter Document List,type,{documentName}, "admin.transport.docs.grid.name_filter"
+110.wait,1000,,
+111. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+112.Click drivers menu,click,, "admin.drivers.menu.icon"
+113.Click Add Driver menu,click,, "admin.drivers.add_menu.link"
+114.Wait For Add Driver, wait_until_visible,, "admin.drivers.add_page.header"
+115.Click Service Category Dropdown,click,, "admin.drivers.service_dropdown.select"
+116.Select Bus Ride Option,click,, "admin.transport.dropdown.dynamic_service"
+117.Enter Driver Name, type, busdriver_{timestamp} &gt;&gt; busDriverName, "admin.drivers.fullname.input"
+118.Enter Email, type, busdriver_{timestamp}@gmail.com&gt;&gt;busEmail, "admin.drivers.email.input"
+119.Enter Contact Number, type, {randomPhone}&gt;&gt;busPhone, "admin.drivers.phone.input"
+120.Click Whatspp,click,, "admin.drivers.whatsapp.checkbox"
+121.Enter Whatspp Number,type,{busPhone}, "admin.drivers.whatsapp_phone.input"
+122.Upload Profile Image, uploadfile, "src/main/resources/test-data/busdriver.jpg", "admin.drivers.profile_image.file"
+123.Select Source,click,, "admin.drivers.source_dropdown.select"
+124.Select Instagram,click,, "admin.drivers.instagram_option.span"
+125.Select Male Gender, click, , "admin.drivers.male_gender.div"
+126.Click Vehicle Type Dropdown,click,, "admin.drivers.vehicle_dropdown.select"
+127.Select  volvo Option,click,, "admin.transport.dropdown.dynamic_vehicle"
+128.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+129.Enter Plate No, type, KL-01-AB-1634, "admin.drivers.plateno.input"
+130. Enter Model Name, type, deisel, "admin.drivers.modelname.input"
+131.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/busvolvo.jpeg", "admin.drivers.vehicle_image.file"
+132.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+133.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
+134.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+135.Enter Account Holder Name, type, {busDriverName}, "admin.drivers.accountholder.input"
+136.Enter Payment Email Address, type, {busEmail}, "admin.drivers.paymentemail.input"
+137.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+138.Click Submit, click, , "web.global.action.submit"
+139.Wait For Driver Added,wait_until_visible, , "web.global.toast.success"
+140.Wait for Toast to hide, wait, 1000,
+141. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+142.Click drivers menu,click,, "admin.drivers.menu.icon"
+143.Click Pending Documents,click,, "admin.drivers.pending_docs.link"
+144.Filter by Name,type,{busDriverName}, "admin.drivers.name_filter.input"
+145.Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+146.Click Doc Icon,click,, "admin.drivers.docs.icon"
+147.Driver Required Documents,verify,, "admin.drivers.required_docs.header"
+148.FilterDocumet List,type,{documentName}, "admin.drivers.docs_filter.input"
+149.Add Driving License,click,, "admin.drivers.docs.edit_icon"
+150.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+151.Enter Expiry Date,type,12-12-2026, "admin.drivers.doc_expiry.input"
+152.Click Submit, click, , "web.global.action.submit"
+153.Wait For Updated Succesfully, wait_until_visible, , "web.global.toast.updated"
+154.Click Approve Driver,click,, "admin.drivers.docs.approval"
+155.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+156. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+157.Click drivers menu,click,, "admin.drivers.menu.icon"
+158.Click Approved Drivers,click,, "admin.drivers.approved_docs.link"
+159.Wait For Approved Drivers List, wait_until_visible,, "admin.drivers.approved_page.header"
+160.Filter Approved Driver,type,{busDriverName}, "admin.drivers.name_filter.input"
+161.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+162.Click Transports Services Menu,click,, "admin.transport.menu.card"
+163.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+164.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+165.Click Edit Icon ,click,, "admin.drivers.docs.edit_icon"
+166.wait,2000,,
+167.Scroll Grid, tab, 5, "admin.transport.name.input"
+168.wait,2000,,
+169.Open status Dropdown,click,, "admin.transport.status.dropdown"
+170.Select Deactivate,click,, "admin.transport.status.deactivate_option"
+171.Click  Submit,click,, "web.global.action.submit"
+172.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+173.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
 2. Click Delivery Services,click,,"admin.deliveryservice.menu"
 3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
@@ -3000,7 +2750,7 @@
 77. wait,1000,,</t>
   </si>
   <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
 2. Click Delivery Services,click,,"admin.deliveryservice.menu"
 3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
@@ -3067,7 +2817,7 @@
 65. wait,1000,,</t>
   </si>
   <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
 2. Click Delivery Services,click,,"admin.deliveryservice.menu"
 3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
@@ -3166,7 +2916,7 @@
 97. wait,1000,,</t>
   </si>
   <si>
-    <t>1.Click badge, click, , "admin.deliveryservice.badge.shield"
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
 2.Click Delivery Services, click, , "admin.deliveryservice.menu"
 3.Verify Delivery Services, verify, , "admin.deliveryservice.header"
 4.Click Add Service Category, click, , "admin.deliveryservice.add_category_btn"
@@ -3307,7 +3057,7 @@
 139.Open Product Category Dropdown, click, , "admin.store.products.category_dropdown"
 140.Select curd, click, , "admin.deliveryservice.products.category.option_dynamic"
 141.wait, 1000, ,""
-142.Click badge, click, , "admin.deliveryservice.badge.shield"
+142.Click Dashboard Icon,click,, "web.global.menu.dashboard"
 143.Click Delivery Services, click, , "admin.deliveryservice.menu"
 144.Verify Delivery Services, verify, , "admin.deliveryservice.header"
 145.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
@@ -3318,6 +3068,255 @@
 150.Click Submit, click, , "web.global.action.submit"
 151.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
 152.wait, 1000, ,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2.Click Delivery Services,click,,"admin.provider_service.menu_link"
+3.Verify Delivery Services,verify,,"admin.provider_service.on_demand_header"
+4.Filter service List,type,Plumbers,"admin.provider_service.services.filter.input"
+5.Click Home Icon Plumbers,click,,"admin.provider_service.services.home.icon_by_row_plumbers"
+6.Verify Plumbers Summary,verify,,"admin.provider_service.services.plumbers_summary.header"
+7.Click Providers,click,,"admin.provider_service.providers.root.button"
+8.Select Add Providers,click,,"admin.provider_service.providers.add_provider.menu"
+9.Verify Add Provider,verify,,"admin.provider_service.provider_form.header"
+10.Enter Provider Full Name, type, Plumber{randomAlpha}&gt;&gt; plumberName, "admin.provider_service.provider_form.fullname.input"
+11.Upload Plumber Image, uploadfile, "src/main/resources/test-data/plumber.jpg", "admin.provider_service.provider_form.avatar.file"
+12.Enter Email, type, Plumber_{timestamp}@gmail.com&gt;&gt;plumberEmail, "admin.provider_service.provider_form.email.input"
+13.Enter Contact Number, type, {randomPhone}, "admin.provider_service.provider_form.contact_number.input"
+14.Enter Landmark, type, Near LIC Building, "admin.provider_service.provider_form.landmark.input"
+15.Open Delivery Radius Dropdown,click,,"admin.provider_service.provider_form.radius.dropdown"
+16.Select Twenty Five Kilometer,click,,"admin.provider_service.provider_form.radius.option_25km"
+17.Enter Minimum Order, type, 10, "admin.provider_service.provider_form.min_order.input"
+18.Enter Provider Address, type, plumber chennai, "admin.provider_service.provider_form.address.input"
+19.wait,1000,,
+20.Select First Option,arrow_down,,"admin.provider_service.provider_form.address.input"
+21.Confirm Option,press_enter,,"admin.provider_service.provider_form.address.input"
+22.wait,1000,,
+23.Click Everyday Checkbox, click, , "admin.provider_service.provider_form.everyday.checkbox"
+24.Click 09:00 AM-10:00 AM, click, , "admin.provider_service.provider_form.time_slot.09_10am"
+25.Click 10:00 AM-11:00 AM, click, , "admin.provider_service.provider_form.time_slot.10_11am"
+26.Click 11:00 AM-12:00 PM, click, , "admin.provider_service.provider_form.time_slot.11_12pm"
+27.Click 12:00 PM-01:00 PM, click, , "admin.provider_service.provider_form.time_slot.12_01pm"
+28.Click 02:00 PM-03:00 PM, click, , "admin.provider_service.provider_form.time_slot.02_03pm"
+29.Click 03:00 PM-04:00 PM, click, , "admin.provider_service.provider_form.time_slot.03_04pm"
+30.Enter Bank Name, type, federal, "admin.provider_service.provider_form.bank_name.input"
+31.Enter Bank Location,type, chennai, "admin.provider_service.provider_form.bank_location.input"
+32.Scroll Grid, tab, 1, "admin.provider_service.provider_form.bank_location.input"
+33.Enter Account Number, type, 123456789012, "admin.provider_service.provider_form.account_number.input"
+34.Enter Account Holder Name, type, {plumberName}, "admin.provider_service.provider_form.account_holder.input"
+35.Enter Payment Email Address, type, {plumberEmail}, "admin.provider_service.provider_form.payment_email.input"
+36.Enter BIC Code, type, 1234, "admin.provider_service.provider_form.bic_code.input"
+37.Click Save, click, , "web.global.login.submit_btn"
+38.Verify Sucess, verify, , "web.global.toast.info"
+39.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+40.Click Providers,click,,"admin.provider_service.providers.root.button"
+41.Select Pending Document Providers,click,,"admin.provider_service.providers.pending_docs.menu"
+42.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+43.Click Document Icon,click,,"admin.provider_service.providers.grid.document.icon"
+44.Provider Required Documents,verify,,"admin.provider_service.provider_docs.header"
+45.FilterDocumet List,type,Store Address,"admin.provider_service.provider_docs.filter.input"
+46.Add Address Proof,click,,"admin.provider_service.provider_docs.edit_action.icon"
+47.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "admin.provider_service.provider_docs.upload_input"
+48.Enter Expiry Date,type,2026-12-12,"admin.provider_service.provider_docs.expiry_date.input"
+49.Click Submit, click, , "web.global.action.submit"
+50.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+51.FilterDocumet List,type,Store Address,"admin.provider_service.provider_docs.filter.input"
+52.Click Approve Store,click,,"admin.provider_service.provider_docs.approve.icon"
+53.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+54.Click Back, click, , "admin.provider_service.global.action.back_widget_btn"
+55.Click Providers,click,,"admin.provider_service.providers.root.button"
+56.Select Provider List,click,,"admin.provider_service.providers.provider_list.menu"
+57.Verify Approved Provider,verify,,"admin.provider_service.providers.grid.approved_plumbers.header"
+58.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+59.Click Doc Icon,click,,"admin.provider_service.providers.grid.document.icon"
+60.Click Eye Icon,click,,"admin.provider_service.providers.grid.view_eye.icon"
+61.Click Back, click, , "admin.provider_service.global.action.back_widget_btn"
+62.Verify Approved Provider,verify,,"admin.provider_service.providers.grid.approved_plumbers.header"
+63.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+64.Scroll Grid, tab, 11, "admin.provider_service.providers.grid.name_filter"
+65.Click Wallet Icon,click,,"admin.provider_service.providers.grid.wallet.icon"
+66.Click Manage Transaction, click, , "admin.provider_service.wallet.manage_transaction.btn"
+67.Enter Wallet Amount, type, 1000, "admin.provider_service.wallet.amount.input"
+68.Open Choose Option Dropdown,click, , "admin.provider_service.wallet.options.dropdown"
+69.Select Add Money,click, , "admin.provider_service.wallet.options.add_money"
+70.Click Submit, click, , "web.global.action.submit"
+71.Verify Saved Succesfully, verify, , "web.global.toast.success"
+72.Click Manage Transaction, click, , "admin.provider_service.wallet.manage_transaction.btn"
+73.Enter Wallet Amount, type, 200, "admin.provider_service.wallet.amount.input"
+74.Open Choose Option Dropdown,click, , "admin.provider_service.wallet.options.dropdown"
+75.Select Deduct Money,click, , "admin.provider_service.wallet.options.deduct_money"
+76.Click Submit, click, , "web.global.action.submit"
+77.Verify Saved Succesfully, verify, , "web.global.toast.success"
+78.Click Back, click, , "admin.provider_service.global.action.back_normal_btn"
+79.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+80.Click Doc Icon,click, , "admin.provider_service.providers.grid.document.icon"
+81.FilterDocumet List,type,Store Address,"admin.provider_service.provider_docs.filter.input"
+82.Click Reject Document,click, , "admin.provider_service.provider_docs.reject.icon"
+83.Click Reject Yes,click, , "web.global.dialog.btn_confirm_yes"
+84.Rejection Reason,type,document insufficent,"web.global.dialog.textarea_reason"
+85..Click Reject Yes,click, , "web.global.dialog.btn_confirm_yes"
+86.Click Back, click, , "admin.provider_service.global.action.back_widget_btn"
+87.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+88.Scroll Grid, tab, 13, "admin.provider_service.providers.grid.name_filter"
+89.Click Block Provider,click, , "admin.provider_service.providers.grid.block.icon"
+90.Click Block Yes,click, , "web.global.dialog.btn_confirm_yes"
+91.Blocking Reason,type,customer complaints,"web.global.dialog.textarea_reason"
+92.Click block Yes,click, , "web.global.dialog.btn_confirm_yes"
+93.Click Providers,click, , "admin.provider_service.providers.root.button"
+94.Select Blocked Providers,click, , "admin.provider_service.providers.blocked_list.menu"
+95.Verify Blocked Provider,verify, , "admin.provider_service.providers.grid.blocked_plumbers.header"
+96.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+97.Scroll Grid, tab, 12, "admin.provider_service.providers.grid.name_filter"
+98.Click Unblock Provider,click, , "admin.provider_service.providers.grid.unblock.icon"
+99.Click Providers,click, , "admin.provider_service.providers.root.button"
+100.Select Provider List,click, , "admin.provider_service.providers.provider_list.menu"
+101.Filter Plumber List,type,{plumberName},"admin.provider_service.providers.grid.name_filter"
+102.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2.Click Provider Services,click,,"admin.provider_service.menu_link"
+3.Verify Provider Services,verify,,"admin.provider_service.on_demand_header"
+4.Click Add New Services,click,,"admin.provider_service.services.add_new.btn"
+5.Enter Service Name, type, Painter{randomAlpha}&gt;&gt; serviceName, "admin.provider_service.services.name.input"
+6.Enter Service Name Tamil, type, பெயிண்டர், "admin.provider_service.services.name_tamil.input"
+7.Enter Service Name Arabic, type, دهان, "admin.provider_service.services.name_arabic.input"
+8.Enter Service Name Hindi, type, पेंटर, "admin.provider_service.services.name_hindi.input"
+9.Enter Slug, type, painter, "admin.provider_service.services.slug.input"
+10.Upload Service Image, uploadfile, "src/main/resources/test-data/painter.jpg", "admin.provider_service.services.image.file"
+11.wait,2000,,
+12.Open status Dropdown,click,,"admin.provider_service.services.status.dropdown"
+13.Select Activate,click,,"admin.provider_service.services.status.option_activate"
+14.Open Select City Dropdown,click,,"admin.provider_service.services.city.dropdown"
+15.Select {areaName},click,,"admin.provider_service.services.city.option_dynamic"
+16.Click Submit,click,,"web.global.action.submit"
+17.Filter Services List,type,{serviceName},"admin.provider_service.services.filter.input"
+18.Click Home Icon ,click,,"admin.provider_service.services.home.icon"
+19.Click Settings ,click,,"admin.provider_service.settings.menu.button"
+20.Click Requirment Document ,click,,"admin.provider_service.settings.req_document.tab"
+21.Click Add Document ,click,,"admin.provider_service.req_docs.add.btn"
+22.Enter Name, type, documet{randomAlpha}&gt;&gt; providerDocumentName, "admin.provider_service.req_docs.name.input"
+23.Open status Dropdown,click,,"admin.provider_service.req_docs.status.dropdown"
+24.Select Active,click,,"admin.provider_service.req_docs.status.option_active"
+25.Click Document Expiry ,click,,"admin.provider_service.req_docs.expiry_toggle"
+26.Click Mandatory Document ,click,,"admin.provider_service.req_docs.mandatory_toggle"
+27.Click Submit ,click,,"web.global.action.submit"
+28.Verify Sucess, verify, , "web.global.toast.info"
+29.Filter Document List,type,{providerDocumentName},"admin.provider_service.req_docs.filter.input"
+30.Click Settings ,click,,"admin.provider_service.settings.menu.button"
+31.Click Promocode ,click,,"admin.provider_service.settings.promocode.tab"
+32.Click Add Promo Code ,click,,"admin.provider_service.promocode.add.btn"
+33.Open User List Dropdown,click,,"admin.provider_service.promocode.user_list.dropdown"
+34.Select User,click,,"admin.provider_service.promocode.user_list.option_dynamic"
+35.Click Code Name Box,click,,"admin.provider_service.promocode.code_name.box"
+36.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; providerPromoCodeName, "admin.provider_service.promocode.code_name.box"
+37.Open Discout Type Dropdown,click,,"admin.provider_service.promocode.discount_type.dropdown"
+38.Select Discout Type,click,,"admin.provider_service.promocode.discount_type.option_amount"
+39.Enter Expiry Date,type,12122026,"admin.provider_service.promocode.expiry_date.input"
+40.Enter Discount Amount, type, 100, "admin.provider_service.promocode.discount_amount.input"
+41.Enter Minimum Order Amount, type, 1000, "admin.provider_service.promocode.min_order_amount.input"
+42.Enter Maximum Discount Amount, type, 100, "admin.provider_service.promocode.max_discount.input"
+43.Enter Coupon Limit, type, 5,"admin.provider_service.promocode.coupon_limit.input"
+44.Enter Usage Limit for One User, type, 2,"admin.provider_service.promocode.usage_limit_per_user.input"
+45.Enter Promo Code Description, type, Promo Dode For Gold Member,"admin.provider_service.promocode.description.textarea"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Verify Sucess, verify, , "web.global.toast.info"
+48.Filter PromoCode List,type,{providerPromoCodeName},"admin.provider_service.promocode.filter.input"
+49.Click Providers,click,,"admin.provider_service.providers.root.button"
+50.Select Add Providers,click,,"admin.provider_service.providers.add_provider.menu"
+51.Verify Add Provider,verify,,"admin.provider_service.provider_form.header"
+52.Enter Provider Full Name, type, Painter{randomAlpha}&gt;&gt; painterName, "admin.provider_service.provider_form.fullname.input"
+53.Upload Painter Image, uploadfile, "src/main/resources/test-data/painter.jpg", "admin.provider_service.provider_form.avatar.file"
+54.Enter Email, type, Painter_{timestamp}@gmail.com&gt;&gt;painterEmail, "admin.provider_service.provider_form.email.input"
+55.Enter Contact Number, type, {randomPhone}, "admin.provider_service.provider_form.contact_number.input"
+56.Enter Landmark, type, Near LIC Building, "admin.provider_service.provider_form.landmark.input"
+57.Open Delivery Radius Dropdown,click,,"admin.provider_service.provider_form.radius.dropdown"
+58.Select Twenty Five Kilometer,click,,"admin.provider_service.provider_form.radius.option_25km"
+59.Enter Minimum Order, type, 10, "admin.provider_service.provider_form.min_order.input"
+60.Enter Provider Address, type, painter chennai, "admin.provider_service.provider_form.address.input"
+61.wait,1000,,
+62.Select First Option,arrow_down,,"admin.provider_service.provider_form.address.input"
+63.Confirm Option,press_enter,,"admin.provider_service.provider_form.address.input"
+64.wait,1000,,
+65.Click Everyday Checkbox, click, , "admin.provider_service.provider_form.everyday.checkbox"
+66.Click 09:00 AM-10:00 AM, click, , "admin.provider_service.provider_form.time_slot.09_10am"
+67.Click 10:00 AM-11:00 AM, click, , "admin.provider_service.provider_form.time_slot.10_11am"
+68.Click 11:00 AM-12:00 PM, click, , "admin.provider_service.provider_form.time_slot.11_12pm"
+69.Click 12:00 PM-01:00 PM, click, , "admin.provider_service.provider_form.time_slot.12_01pm"
+70.Click 02:00 PM-03:00 PM, click, , "admin.provider_service.provider_form.time_slot.02_03pm"
+71.Click 03:00 PM-04:00 PM, click, , "admin.provider_service.provider_form.time_slot.03_04pm"
+72.Enter Bank Name, type, federal, "admin.provider_service.provider_form.bank_name.input"
+73.Enter Bank Location,type, chennai, "admin.provider_service.provider_form.bank_location.input"
+74.Scroll Grid, tab, 1, "admin.provider_service.provider_form.bank_location.input"
+75.Enter Account Number, type, 123456789012, "admin.provider_service.provider_form.account_number.input"
+76.Enter Accont Holder Name, type, {painterName}, "admin.provider_service.provider_form.account_holder.input"
+77.Enter Payment Email Address, type, {painterEmail}, "admin.provider_service.provider_form.payment_email.input"
+78.Enter BIC Code, type, 1234, "admin.provider_service.provider_form.bic_code.input"
+79.Click Save, click, , "web.global.login.submit_btn"
+80.Verify Sucess, verify, , "web.global.toast.info"
+81.Filter Painter List,type,{painterName},"admin.provider_service.providers.grid.name_filter"
+82.Click Providers,click,,"admin.provider_service.providers.root.button"
+83.Select Pending Document Providers,click,,"admin.provider_service.providers.pending_docs.menu"
+84.Filter Plumber List,type,{painterName},"admin.provider_service.providers.grid.name_filter"
+85.Click Document Icon,click,,"admin.provider_service.providers.grid.document.icon"
+86.Provider Required Documents,verify,,"admin.provider_service.provider_docs.header"
+87.FilterDocumet List,type,{providerDocumentName},"admin.provider_service.provider_docs.filter.input"
+88.Add Address Proof,click,,"admin.provider_service.provider_docs.edit_action.icon"
+89.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "admin.provider_service.provider_docs.upload_input"
+90.Enter Expiry Date,type,2026-12-12,"admin.provider_service.provider_docs.expiry_date.input"
+91.Click Submit, click, , "web.global.action.submit"
+92.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+93.FilterDocumet List,type,{providerDocumentName},"admin.provider_service.provider_docs.filter.input"
+94.Click Approve Store,click,,"admin.provider_service.provider_docs.approve.icon"
+95.Verify Updated Succesfully, verify, , "web.global.toast.updated"
+96.Click Back, click, , "admin.provider_service.global.action.back_widget_btn"
+97.Click Providers,click,,"admin.provider_service.products.menu_category_btn"
+98.Click Add New Category,click,,"admin.provider_service.category.add_new.btn"
+99.Enter Category Name, type,residentialPainter{randomAlpha}&gt;&gt; painterCategoryName, "admin.provider_service.category.name.input"
+100.Enter Category Name Tamil, type, குடியிருப்பு பெயிண்டர், "admin.provider_service.category.name_tamil.input"
+101.Enter Category Name Arabic, type, دهان سكني, "admin.provider_service.category.name_arabic.input"
+102.Enter Category Name Hindi, type, आवासीय पेंटर, "admin.provider_service.category.name_hindi.input"
+103.Open Category status Dropdown,click,,"admin.provider_service.category.status.dropdown"
+104.Select Activate,click,,"admin.provider_service.category.status.option_active"
+105.Upload Category Image, uploadfile, "src/main/resources/test-data/painter.jpg", "admin.provider_service.category.image.file"
+106.wait,2000,,
+107.Click Submit,click,,"web.global.action.submit"
+108.Filter Category Name,type,{painterCategoryName},"admin.provider_service.category.filter.input"
+109.Click Providers,click,,"admin.provider_service.providers.root.button"
+110.Select Provider List,click,,"admin.provider_service.providers.provider_list.menu"
+111.Filter Painter List,type,{painterName},"admin.provider_service.providers.grid.name_filter"
+112.Scroll Grid, tab, 7, "admin.provider_service.providers.grid.name_filter"
+113.Click Package Icon,click,,"admin.provider_service.packages.icon"
+114.Click Add Package,click,,"admin.provider_service.packages.add_new.btn"
+115.Open Category Dropdown,click,,"admin.provider_service.packages.category.dropdown"
+116.Select Activate,click,,"admin.provider_service.packages.category.option_dynamic"
+117.Enter Package Name, type, package{randomAlpha}&gt;&gt; packageName, "admin.provider_service.packages.name.input"
+118.Enter Amount, type, 1000, "admin.provider_service.packages.amount.input"
+119.Open Max Book Quantity Dropdown,click,,"admin.provider_service.packages.max_book_qty.dropdown"
+120.Select 4,click,,"admin.provider_service.packages.max_book_qty.option_4"
+121.Open Status Dropdown,click,,"admin.provider_service.packages.status.dropdown"
+122.Select Activate,click,,"admin.provider_service.packages.status.option_activate"
+123.Enter Description, type, Premium residential painting package, "admin.provider_service.packages.description.textarea"
+124.Click Submit,click,,"web.global.action.submit"
+125.wait,1000,,
+126.Click back,click,,"admin.provider_service.global.action.back_normal_btn"
+127.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+128.Click Delivery Services,click,,"admin.provider_service.menu_link"
+129.Filter Services List,type,{serviceName},"admin.provider_service.services.filter.input"
+130.Click Edit Icon ,click,,"admin.provider_service.services.edit.icon"
+131.Enter Service Name Tamil, type, பெயிண்டர், "admin.provider_service.services.name_tamil.input"
+132.Enter Service Name Arabic, type, دهان, "admin.provider_service.services.name_arabic.input"
+133.Enter Service Name Hindi, type, पेंटर, "admin.provider_service.services.name_hindi.input"
+134.Scroll Grid, tab, 4, "admin.provider_service.services.name_hindi.input"
+135.Open status Dropdown,click,,"admin.provider_service.services.status.dropdown"
+136.Select Deactivate,click,,"admin.provider_service.services.status.option_deactivate"
+137.Click Submit,click,,"web.global.action.submit"
+138.Click back,click,,"admin.provider_service.global.action.back_normal_btn"
+139. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+140.Click badge,click,,"admin.provider_service.badge.icon"
+141.Click provider Services,click,,"admin.provider_service.menu_link"
+142.Filter Services List,type,{serviceName},"admin.provider_service.services.filter.input"
+143.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -3734,7 +3733,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3743,7 +3742,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -3812,13 +3811,13 @@
         <v>27</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3884,16 +3883,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3956,13 +3955,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -4015,36 +4014,36 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="G2" s="8" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4060,7 +4059,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF16C04E-51BB-4902-91C6-410B8EB3791F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4101,19 +4100,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -4132,7 +4131,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E742ED82-3510-47F4-AA85-6344770C749C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4173,22 +4172,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4204,7 +4203,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6277B-DBCF-4BFF-819C-1E90748D3258}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F69F54-6E80-4C66-8F82-CEFA135D089A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4245,22 +4244,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4317,22 +4316,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4384,7 +4383,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4404,13 +4403,13 @@
         <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4483,7 +4482,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -4538,7 +4537,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4558,13 +4557,13 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -4606,7 +4605,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4620,19 +4619,19 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4681,7 +4680,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4695,19 +4694,19 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4756,7 +4755,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4770,19 +4769,19 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4831,7 +4830,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4842,22 +4841,22 @@
         <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4915,22 +4914,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
86th Commit: Click If Present Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CD8D22-D938-471C-9746-0A3DAF50DB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2CD1B2E-433C-4905-B32A-49654B080792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="18" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="19" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -25,16 +25,18 @@
     <sheet name="TransportServiceStatisticsTest" sheetId="51" r:id="rId10"/>
     <sheet name="TransportDriverStatisticsTest" sheetId="52" r:id="rId11"/>
     <sheet name="TransportServiceRidesTest" sheetId="53" r:id="rId12"/>
-    <sheet name="SubscriptionPlanTest" sheetId="47" r:id="rId13"/>
-    <sheet name="PanicCallTest" sheetId="49" r:id="rId14"/>
-    <sheet name="DashboardTest" sheetId="50" r:id="rId15"/>
-    <sheet name="AddStore" sheetId="40" r:id="rId16"/>
-    <sheet name="StoreOperations" sheetId="42" r:id="rId17"/>
-    <sheet name="StoreStatusManagement" sheetId="43" r:id="rId18"/>
-    <sheet name="DeliveryServiceCompleteTest" sheetId="44" r:id="rId19"/>
-    <sheet name="AddProvider" sheetId="45" r:id="rId20"/>
-    <sheet name="ProviderServiceCompleteTest" sheetId="46" r:id="rId21"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId22"/>
+    <sheet name="TransportServiceAerialView" sheetId="54" r:id="rId13"/>
+    <sheet name="SubscriptionPlanTest" sheetId="47" r:id="rId14"/>
+    <sheet name="PanicCallTest" sheetId="49" r:id="rId15"/>
+    <sheet name="DashboardTest" sheetId="50" r:id="rId16"/>
+    <sheet name="AddStore" sheetId="40" r:id="rId17"/>
+    <sheet name="StoreOperations" sheetId="42" r:id="rId18"/>
+    <sheet name="StoreStatusManagement" sheetId="43" r:id="rId19"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="44" r:id="rId20"/>
+    <sheet name="AddProvider" sheetId="45" r:id="rId21"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="46" r:id="rId22"/>
+    <sheet name="DEMO" sheetId="55" r:id="rId23"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId24"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="151">
   <si>
     <t>City Area</t>
   </si>
@@ -3163,9 +3165,6 @@
     <t>SA_TS_21</t>
   </si>
   <si>
-    <t>TC_CA_21_test_data_cleanup</t>
-  </si>
-  <si>
     <t>This end-to-end regression test suite thoroughly validates the data filtering, search capabilities, and transaction monitoring matrices within the Transport Services administration panel. The test starts by targeting a specific vehicle class ("Auto Ride") and systematically loops through chronological milestone filters—ranging from Today to Last Year—to verify date-partitioned metrics rendering. It then transitions to a complex granular query verification phase by isolating discrete parameters across multiple dependent dropdown elements, including specific customer names, registered driver profiles, vehicle types ("Pink Auto"), and ride lifecycles (Completed, Incomplete, Cancelled, Scheduled, and Pre-Acceptance Cancel Rides). Additionally, the script tests contextual UI elements by verifying the operational initialization of intra-ride chat boxes and auditing specialized tracking panels, such as arrival time breakdowns and deep-dive ride detail metrics grids, ensuring robust data reporting with zero caching conflicts across state changes.</t>
   </si>
   <si>
@@ -3554,31 +3553,285 @@
     <t>TC_CA_11_Transport_Service_Ride_Test</t>
   </si>
   <si>
-    <t>TC_CA_12_subscription_plan_test</t>
-  </si>
-  <si>
-    <t>TC_CA_13_Panic_Call_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_14_Dashboard_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_15_add_store</t>
-  </si>
-  <si>
-    <t>TC_CA_16_store_oprerations</t>
-  </si>
-  <si>
-    <t>TC_CA_17_store_status_management</t>
-  </si>
-  <si>
-    <t>TC_CA_18_delivery_service_complete_test</t>
-  </si>
-  <si>
-    <t>TC_CA_19_add_provider</t>
-  </si>
-  <si>
-    <t>TC_CA_20_provider_service_full_lifecycle_test</t>
+    <t xml:space="preserve">1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2. Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Filter Services List,type,Auto Ride, "admin.transport.grid.name_filter"
+4.Click Home Icon,Click,,"admin.transport.home.icon"
+5.Click AerialView Button,click,,"admin.transport.aerial_view.top_menu_btn"
+6.Click All Button,click,,"admin.transport.aerial_view.submenu_all_btn"
+7.Click Eye Button,click_if_present,,"admin.transport.aerial_view.eye_icon"
+8.Click Popup Close Button,click_if_present,,"admin.transport.aerial_view.eye_icon_close"
+9.Click AerialView Button,click,,"admin.transport.aerial_view.top_menu_btn"
+10.Click available button,click,,"admin.transport.aerial_view.submenu_available_btn"
+11.Click Eye Button,click_if_present,,"admin.transport.aerial_view.eye_icon"
+12.Click Popup Close Button,click_if_present,,"admin.transport.aerial_view.eye_icon_close"
+13.Click AerialView Button,click,,"admin.transport.aerial_view.top_menu_btn"
+14.Click Enroute to pickup,click,,"admin.transport.aerial_view.submenu_enroute_pickup_btn"
+15.Click Eye Button,click_if_present,,"admin.transport.aerial_view.eye_icon"
+16.Click Popup Close Button,click_if_present,,"admin.transport.aerial_view.eye_icon_close"
+17.Click AerialView Button,click,,"admin.transport.aerial_view.top_menu_btn"
+18.Click Reached Pickup,click,,"admin.transport.aerial_view.submenu_reached_pickup_btn"
+19.Click Eye Button,click_if_present,,"admin.transport.aerial_view.eye_icon"
+20.Click Popup Close Button,click_if_present,,"admin.transport.aerial_view.eye_icon_close"
+21.Click AerialView Button,click,,"admin.transport.aerial_view.top_menu_btn"
+22.Click Ongoing Button,click,,"admin.transport.aerial_view.submenu_ongoing_btn"
+23.Click Eye Button,click_if_present,,"admin.transport.aerial_view.eye_icon"
+24.Click Popup Close Button,click_if_present,,"admin.transport.aerial_view.eye_icon_close"
+</t>
+  </si>
+  <si>
+    <t>Transport Service Aerial View</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet:SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>This targeted regression test suite validates the operational map metrics and driver tracking grids within the Transport Services Aerial View monitoring control center. The test targets a specific service class ("Auto Ride") and systematically loops through all real-time operational filters in the geospatial dashboard—specifically auditing the telemetry statuses for All, Available, Enroute to Pickup, Reached Pickup, and Ongoing tracking segments. For each individual status layout, the script uses the fault-tolerant click_if_present keyword to launch detailed map overlay info-popups via the tracking eye icon, verifies panel readability, and dismisses the popup cleanly before moving to the next status. This process ensures that dynamic map layers, dispatcher tooltips, and real-time operational status updates function flawlessly across the administrative workspace without crashing due to unexpected timing or missing elements.</t>
+  </si>
+  <si>
+    <t>TC_CA_12_Transport_Service_Aerial_View</t>
+  </si>
+  <si>
+    <t>TC_CA_13_subscription_plan_test</t>
+  </si>
+  <si>
+    <t>TC_CA_14_Panic_Call_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_15_Dashboard_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_16_add_store</t>
+  </si>
+  <si>
+    <t>TC_CA_17_store_oprerations</t>
+  </si>
+  <si>
+    <t>TC_CA_18_store_status_management</t>
+  </si>
+  <si>
+    <t>TC_CA_19_delivery_service_complete_test</t>
+  </si>
+  <si>
+    <t>TC_CA_20_add_provider</t>
+  </si>
+  <si>
+    <t>TC_CA_21_provider_service_full_lifecycle_test</t>
+  </si>
+  <si>
+    <t>SA_TS_22</t>
+  </si>
+  <si>
+    <t>TC_CA_22_test_data_cleanup</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Provider and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_CA_XX_Demo</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2.Click Transport Service,Click,,"//h2[@id='Transport Services']"
+3.Click Search Box,click,,"//input[@class='ag-input-field-input ag-text-field-input']"
+4.Enter Services,type,Auto Ride,"//input[@class='ag-input-field-input ag-text-field-input']"
+5.Click Home Icon,Click,,"//i[@title='Home']"
+6.Click Earning Report,click,,"//button[text()=" Earnings Reports "]"
+7.Click Today Button,Click,,"//button[normalize-space()='Today']"
+8.Click Yesterday Button,Click,,"//button[normalize-space()='Yesterday']"
+9.Click This Week Button,Click,,"//button[normalize-space()='This Week']"
+10.Click This Month Button,Click,,"//button[normalize-space()='This Month']"
+11.Click Last Month Button,Click,,"//button[normalize-space()='Last Month']"
+12.Click This Year Button,Click,,"//button[normalize-space()='This Year']"
+13.Click Last Year Button,Click,,"//button[normalize-space()='Last Year']"
+14.Click This Year Button,Click,,"//button[normalize-space()='This Year']"
+15.Click Driver dropdown,click,,"//div[@id='Select Driver']//span[@role='combobox']"
+16.Click Search Name,click,,"//input[@role='searchbox']"
+17.Search Driver Name,type,sujan pariyar,"//input[@role='searchbox']" 
+18.Click Driver Name,click,,"//li[@role='option' and @aria-label='Sujan Pariyar A']"
+19.Click Customer Search Dropdown,click,,"//div[@id='Select Customer']"
+20.Click Search Box,click,,"//input[@role='searchbox']"
+21.Search Customer name,type,mohamed yasir,"//input[@role='searchbox']"
+22.Select The Customer,click,,"//li[@id='Select Customer_0']//span[@class='ng-star-inserted']"
+23.Click payment type,click,,"//div[@id='Select Payment Type']"
+24.Click Select cash Payment Type,click,,"//li[@id='Select Payment Type_0']"
+25.Click payment type,click,,"//div[@id='Select Payment Type']"
+26.Click Razor Payment,click,,"//li[@id='Select Payment Type_1']"
+27.Click payment type,click,,"//div[@id='Select Payment Type']"
+28.Click wallet option,click,,"//li[@id='Select Payment Type_2']"
+29.Click payment type,click,,"//div[@id='Select Payment Type']"
+30.Click Select cash Payment Type,click,,"//li[@id='Select Payment Type_0']"
+31.Click Driver Payment Status,click,,"//div[@id='Select Driver Payment Status']"
+32.Click Settled Button,click,,"//li[@role='option' and @aria-label='Settled']"
+33.Click Driver Payment Status,click,,"//div[@id='Select Driver Payment Status']"
+34.Click Unsettled Button,click,,"//li[@role='option' and @aria-label='Unsettled']"
+35.Click Search Button,click,,"//button[normalize-space()='Search']
+36.Click Clear Button,click,,"//button[normalize-space()='Clear']"
+37.Click payment type,click,,"//div[@id='Select Payment Type']"
+38.Click Select cash Payment Type,click,,"//li[@id='Select Payment Type_0']"
+39.Click Driver Payment Status,click,,"//div[@id='Select Driver Payment Status']"
+40.Click Unsettled Button,click,,"//li[@role='option' and @aria-label='Unsettled']"
+41.Click Search Button,click,,"//button[normalize-space()='Search']
+42.Click Check Box,click,,"//input[@id='ag-13832-input']"
+43.Click Payment StatusFilter,click,,"//input[@aria-label='Payment Status Filter Input']"
+44.Scroll Grid,tab,24,"//input[@aria-label='Payment Status Filter Input']"
+45.Click Eye Button,Click,,"//i[@title='View']"
+46.Click Mark As Settle Button,click,,"//button[normalize-space()='Mark As Settle']"</t>
   </si>
 </sst>
 </file>
@@ -3992,7 +4245,7 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>62</v>
@@ -4067,13 +4320,13 @@
     </row>
     <row r="2" spans="1:8" ht="360" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>108</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>109</v>
@@ -4145,7 +4398,7 @@
         <v>113</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>112</v>
@@ -4217,10 +4470,10 @@
         <v>115</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>117</v>
@@ -4242,6 +4495,78 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705BF950-38CF-4525-A333-E60DE1739EA0}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F69F54-6E80-4C66-8F82-CEFA135D089A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4283,19 +4608,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>61</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>60</v>
@@ -4313,7 +4638,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB09688-59B4-47C6-9CAD-FED2B503D101}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4355,13 +4680,13 @@
     </row>
     <row r="2" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>99</v>
@@ -4385,7 +4710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23692DF2-D92E-4735-942F-857C385D78E2}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4427,13 +4752,13 @@
     </row>
     <row r="2" spans="1:8" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>106</v>
@@ -4457,7 +4782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9950CA5-B845-4E23-9843-8D459D399E99}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4499,13 +4824,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
@@ -4529,7 +4854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE0E168-E98A-49FE-8885-7B5F3F3678F3}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4571,13 +4896,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -4601,7 +4926,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9584B63-AFDB-41EC-A160-356B47922D15}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4643,13 +4968,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
@@ -4659,85 +4984,6 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A1C6E6-1358-42F0-B7B3-06420689DEE4}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="44.33203125" customWidth="1"/>
-    <col min="8" max="8" width="27.109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4795,7 +5041,7 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
@@ -4832,6 +5078,85 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A1C6E6-1358-42F0-B7B3-06420689DEE4}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="44.33203125" customWidth="1"/>
+    <col min="8" max="8" width="27.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF16C04E-51BB-4902-91C6-410B8EB3791F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4873,13 +5198,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>27</v>
@@ -4903,7 +5228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E742ED82-3510-47F4-AA85-6344770C749C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4945,13 +5270,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>46</v>
@@ -4975,7 +5300,79 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4B640C4-00BD-478A-A57E-A90215D007C2}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5017,19 +5414,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>57</v>
@@ -5092,7 +5489,7 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -5167,7 +5564,7 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
@@ -5235,7 +5632,7 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>10</v>
@@ -5310,7 +5707,7 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>11</v>
@@ -5385,7 +5782,7 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
@@ -5460,7 +5857,7 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>50</v>
@@ -5472,7 +5869,7 @@
         <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
98th Commit: Main Engine Configured For New Excel Format
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512B79EF-7F04-4A2C-A84C-EFB163308031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B200E7-37B5-47FB-B4D4-D6F24856E45A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="185">
   <si>
     <t>City Area</t>
   </si>
@@ -4227,6 +4227,9 @@
 59.Wait For View,wait,200,
 60.Close Earning Report View,click,,"admin.transport.earning_reports.eye_btn_close"
 61.Wait For Close,wait,2000,</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
   </si>
 </sst>
 </file>
@@ -4620,7 +4623,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>184</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>

</xml_diff>